<commit_message>
Interface web, périmètre client par nommage et comparatif Zabbix par API
- Filtre client sur le nommage des hôtes et services (chaînes, regex,
  exclusions, mode et/ou), clients enregistrés et préfixes détectés.
- Inventaire Zabbix par l'API JSON-RPC (5.0 à 7.x, jeton ou login,
  lecture seule) et comparatif : hôtes présents/absents, templates à
  lier ou à importer, statut Zabbix de chaque service, hôtes uniquement
  dans Zabbix.
- Interface web Flask : extractions Centreon/Zabbix, tableau de bord,
  tableaux filtrables, saisie des décisions propagées aux services,
  export Excel du périmètre. Secrets jamais enregistrés, auth Basic
  optionnelle.
- Décisions persistées et reportées dans l'Excel ; options CLI
  équivalentes (--client-*, --zabbix-*, --decisions).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ss1AXzb7kQY6cySve132CB
</commit_message>
<xml_diff>
--- a/examples/matrice_exemple.xlsx
+++ b/examples/matrice_exemple.xlsx
@@ -14,15 +14,21 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Services" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Croisé hôtes x tpl hôtes" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Croisé hôtes x tpl services" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commandes" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparatif Zabbix hôtes" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Uniquement dans Zabbix" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Templates Zabbix" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commandes" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Matrice templates services'!$A$1:$AA$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matrice templates hôtes'!$A$1:$R$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Matrice templates services'!$A$1:$AB$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matrice templates hôtes'!$A$1:$S$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Hôtes'!$A$1:$Q$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Services'!$A$1:$V$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Commandes'!$A$1:$G$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Services'!$A$1:$X$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Comparatif Zabbix hôtes'!$A$1:$Q$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Uniquement dans Zabbix'!$A$1:$H$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Templates Zabbix'!$A$1:$E$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Commandes'!$A$1:$G$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -114,7 +120,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="9">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -154,6 +160,13 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00EDEDED"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00F8CBAD"/>
         </patternFill>
       </fill>
     </dxf>
@@ -533,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -553,7 +566,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Généré le 15/10/2026 12:58</t>
+          <t>Généré le 15/10/2026 14:45</t>
         </is>
       </c>
     </row>
@@ -912,370 +925,1546 @@
         <v>1</v>
       </c>
     </row>
+    <row r="40"/>
     <row r="41">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>Top 15 des templates de service (par nombre de services)</t>
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Zabbix</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>https://zabbix.demo.local (version 7.0.5)</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>Template de service</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Nb services</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Nb hôtes</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>Proposition</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>Template Zabbix suggéré</t>
-        </is>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Hôtes Zabbix</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Base-Ping-LAN</t>
+          <t>Templates Zabbix</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>5</v>
-      </c>
-      <c r="C43" t="n">
-        <v>5</v>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Migrer (template natif)</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>ICMP Ping</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>OS-Linux-Memory-SNMP-custom</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>5</v>
-      </c>
-      <c r="C44" t="n">
-        <v>4</v>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Migrer (template natif)</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Linux by SNMP</t>
-        </is>
-      </c>
-    </row>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="44"/>
     <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>OS-Linux-Cpu-SNMP-custom</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>4</v>
-      </c>
-      <c r="C45" t="n">
-        <v>4</v>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Migrer (template natif)</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Linux by SNMP</t>
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Hôtes Centreon par statut Zabbix</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Nb hôtes</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>OS-Linux-Disk-Generic-Name-SNMP-custom</t>
+          <t>Absent de Zabbix</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>3</v>
-      </c>
-      <c r="C46" t="n">
-        <v>3</v>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Migrer (template natif)</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Linux by SNMP</t>
-        </is>
+        <v>5</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>App-Protocol-HTTP-Response-Time-custom</t>
+          <t>Présent – templates à lier</t>
         </is>
       </c>
       <c r="B47" t="n">
         <v>2</v>
       </c>
-      <c r="C47" t="n">
-        <v>2</v>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Migrer (adapter)</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Website by Browser</t>
-        </is>
-      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>App-Webserver-Apache-Requests-custom</t>
+          <t>Présent – templates OK</t>
         </is>
       </c>
       <c r="B48" t="n">
         <v>2</v>
       </c>
-      <c r="C48" t="n">
-        <v>2</v>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>Migrer (template natif)</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Apache by HTTP</t>
-        </is>
-      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ERP-Batch-Nocturne</t>
+          <t>Hôtes uniquement dans Zabbix</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>2</v>
-      </c>
-      <c r="C49" t="n">
         <v>1</v>
       </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>À analyser</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Net-Cisco-Standard-Environment-SNMP-custom</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>2</v>
-      </c>
-      <c r="C50" t="n">
-        <v>2</v>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Migrer (template natif)</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>(template constructeur SNMP)</t>
-        </is>
-      </c>
-    </row>
+    </row>
+    <row r="50"/>
     <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>OS-Windows-Cpu-SNMP-custom</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>2</v>
-      </c>
-      <c r="C51" t="n">
-        <v>2</v>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Migrer (template natif)</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Windows by SNMP</t>
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Services Centreon par statut Zabbix</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Nb services</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>OS-Windows-Disk-Generic-Name-SNMP-custom</t>
+          <t>Hôte absent de Zabbix</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>2</v>
-      </c>
-      <c r="C52" t="n">
-        <v>2</v>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Migrer (template natif)</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Windows by SNMP</t>
-        </is>
+        <v>15</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>(aucun template) check_erp_batch</t>
+          <t>Couvert dans Zabbix</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>1</v>
-      </c>
-      <c r="C53" t="n">
-        <v>1</v>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>À analyser</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr"/>
+        <v>9</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>App-DB-MySQL-Connection-Time-custom</t>
+          <t>Template à lier</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>1</v>
-      </c>
-      <c r="C54" t="n">
-        <v>1</v>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Migrer (template natif)</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>MySQL by Zabbix agent 2</t>
-        </is>
+        <v>5</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Net-Cisco-Standard-Traffic-Generic-Name-SNMP-custom</t>
+          <t>À créer dans Zabbix</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>1</v>
-      </c>
-      <c r="C55" t="n">
-        <v>1</v>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>Migrer (template natif)</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>(template constructeur SNMP)</t>
-        </is>
+        <v>3</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>Non migré (décision)</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>Top 15 des templates de service (par nombre de services)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Template de service</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Nb services</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Nb hôtes</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Proposition</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>Template Zabbix suggéré</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Base-Ping-LAN</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>5</v>
+      </c>
+      <c r="C60" t="n">
+        <v>5</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>ICMP Ping</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>OS-Linux-Memory-SNMP-custom</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>5</v>
+      </c>
+      <c r="C61" t="n">
+        <v>4</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Linux by SNMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>OS-Linux-Cpu-SNMP-custom</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>4</v>
+      </c>
+      <c r="C62" t="n">
+        <v>4</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Linux by SNMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>OS-Linux-Disk-Generic-Name-SNMP-custom</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>3</v>
+      </c>
+      <c r="C63" t="n">
+        <v>3</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Linux by SNMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>App-Protocol-HTTP-Response-Time-custom</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>2</v>
+      </c>
+      <c r="C64" t="n">
+        <v>2</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Migrer (adapter)</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Website by Browser</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>App-Webserver-Apache-Requests-custom</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>2</v>
+      </c>
+      <c r="C65" t="n">
+        <v>2</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Apache by HTTP</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>ERP-Batch-Nocturne</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>2</v>
+      </c>
+      <c r="C66" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>À analyser</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Net-Cisco-Standard-Environment-SNMP-custom</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>2</v>
+      </c>
+      <c r="C67" t="n">
+        <v>2</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>(template constructeur SNMP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>OS-Windows-Cpu-SNMP-custom</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>2</v>
+      </c>
+      <c r="C68" t="n">
+        <v>2</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Windows by SNMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>OS-Windows-Disk-Generic-Name-SNMP-custom</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>2</v>
+      </c>
+      <c r="C69" t="n">
+        <v>2</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Windows by SNMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>(aucun template) check_erp_batch</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>1</v>
+      </c>
+      <c r="C70" t="n">
+        <v>1</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>À analyser</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>App-DB-MySQL-Connection-Time-custom</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>1</v>
+      </c>
+      <c r="C71" t="n">
+        <v>1</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>MySQL by Zabbix agent 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Net-Cisco-Standard-Traffic-Generic-Name-SNMP-custom</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>1</v>
+      </c>
+      <c r="C72" t="n">
+        <v>1</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>(template constructeur SNMP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
           <t>OS-Linux-Process-Generic-SNMP-custom</t>
         </is>
       </c>
-      <c r="B56" t="n">
+      <c r="B73" t="n">
         <v>1</v>
       </c>
-      <c r="C56" t="n">
+      <c r="C73" t="n">
         <v>1</v>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D73" t="inlineStr">
         <is>
           <t>Migrer (adapter)</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="E73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
         <is>
           <t>OS-Windows-Services-NRPE-custom</t>
         </is>
       </c>
-      <c r="B57" t="n">
+      <c r="B74" t="n">
         <v>1</v>
       </c>
-      <c r="C57" t="n">
+      <c r="C74" t="n">
         <v>1</v>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D74" t="inlineStr">
         <is>
           <t>Migrer (template natif)</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="E74" t="inlineStr">
         <is>
           <t>Windows by Zabbix agent</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="33" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Template Zabbix suggéré</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Disponible dans Zabbix</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Nom technique Zabbix</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Nb hôtes Zabbix liés</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Utilisations Centreon (hôtes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Linux by SNMP</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Linux by SNMP</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Windows by SNMP</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Windows by SNMP</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ICMP Ping</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ICMP Ping</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Apache by HTTP</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Apache by HTTP</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Cisco IOS by SNMP</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Cisco IOS by SNMP</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>MySQL by Zabbix agent 2</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MySQL by Zabbix agent 2</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Website by Browser</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Non (à importer)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Windows by Zabbix agent</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Windows by Zabbix agent</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>APC UPS by SNMP</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Non (à importer)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E10"/>
+  <conditionalFormatting sqref="B2:B10">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>B2="Présent – templates OK"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>B2="Couvert dans Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="4">
+      <formula>B2="Présent – templates à lier"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="4">
+      <formula>B2="Template à lier"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="1">
+      <formula>B2="Présent"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="6">
+      <formula>B2="Absent de Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" dxfId="6">
+      <formula>B2="Hôte absent de Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="2">
+      <formula>B2="À créer dans Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="9" dxfId="3">
+      <formula>B2="Non migré (décision)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="6">
+      <formula>B2="Non (à importer)"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="90" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Commande</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Exécutable</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Plugin</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Mode</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Nb services</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Ligne de commande</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>App-DB-MySQL-Connections</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>centreon_mysql.pl</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>database::mysql::plugin</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>connection-time</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>$CENTREONPLUGINS$/centreon_mysql.pl --plugin=database::mysql::plugin --mode=connection-time --host=$HOSTADDRESS$ --username='$_HOSTMYSQLUSERNAME$' --password=********</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>App-Monitoring-Centreon-Ping</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>check_icmp</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>$USER1$/check_icmp -H $HOSTADDRESS$ -n $_SERVICEPACKETNUMBER$ -w $_SERVICEWARNING$ -c $_SERVICECRITICAL$</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>App-Protocol-HTTP-Response</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>centreon_protocol_http.pl</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>apps::protocols::http::plugin</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>$CENTREONPLUGINS$/centreon_protocol_http.pl --plugin=apps::protocols::http::plugin --mode=response --hostname=$_SERVICEURLHOST$ --urlpath='$_SERVICEURLPATH$' --ssl-opt='SSL_verify_mode =&gt; SSL_VERIFY_NONE'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>App-Webserver-Apache-Requests</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>centreon_apache_serverstatus.pl</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>apps::apache::serverstatus::plugin</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>requests</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>$CENTREONPLUGINS$/centreon_apache_serverstatus.pl --plugin=apps::apache::serverstatus::plugin --mode=requests --hostname=$HOSTADDRESS$</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>base_host_alive</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>check_icmp</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>$USER1$/check_icmp -H $HOSTADDRESS$ -w 3000.0,80% -c 5000.0,100% -p 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>check_centreon_dummy</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>check_dummy</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>$USER1$/check_dummy -o $ARG1$ -s $ARG2$</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>check_erp_batch</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>check_erp_batch.sh</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>$USER2$/check_erp_batch.sh -H $HOSTADDRESS$ -j $ARG1$ -w $ARG2$ -c $ARG3$</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Net-Cisco-Standard-SNMP-Environment</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>centreon_cisco_standard_snmp.pl</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>network::cisco::standard::snmp::plugin</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>environment</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>$CENTREONPLUGINS$/centreon_cisco_standard_snmp.pl --plugin=network::cisco::standard::snmp::plugin --mode=environment --hostname=$HOSTADDRESS$ --snmp-community=********</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Net-Cisco-Standard-SNMP-Traffic-Name</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>centreon_cisco_standard_snmp.pl</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>network::cisco::standard::snmp::plugin</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>interfaces</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>$CENTREONPLUGINS$/centreon_cisco_standard_snmp.pl --plugin=network::cisco::standard::snmp::plugin --mode=interfaces --hostname=$HOSTADDRESS$ --snmp-community=******** --interface='$_SERVICEINTERFACENAME$' --name</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>OS-Linux-SNMP-Cpu</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>centreon_linux_snmp.pl</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>os::linux::snmp::plugin</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>4</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>$CENTREONPLUGINS$/centreon_linux_snmp.pl --plugin=os::linux::snmp::plugin --mode=cpu --hostname=$HOSTADDRESS$ --snmp-version='$_HOSTSNMPVERSION$' --snmp-community=******** --warning-average='$_SERVICEWARNING$' --critical-average='$_SERVICECRITICAL$'</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>OS-Linux-SNMP-Disk-Name</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>centreon_linux_snmp.pl</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>os::linux::snmp::plugin</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>storage</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>3</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>$CENTREONPLUGINS$/centreon_linux_snmp.pl --plugin=os::linux::snmp::plugin --mode=storage --hostname=$HOSTADDRESS$ --snmp-version='$_HOSTSNMPVERSION$' --snmp-community=******** --storage='$_SERVICEDISKNAME$' --name --warning-usage='$_SERVICEWARNING$' --critical-usage='$_SERVICECRITICAL$'</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>OS-Linux-SNMP-Memory</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>centreon_linux_snmp.pl</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>os::linux::snmp::plugin</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>memory</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>5</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>$CENTREONPLUGINS$/centreon_linux_snmp.pl --plugin=os::linux::snmp::plugin --mode=memory --hostname=$HOSTADDRESS$ --snmp-version='$_HOSTSNMPVERSION$' --snmp-community=******** --warning-usage='$_SERVICEWARNING$' --critical-usage='$_SERVICECRITICAL$'</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>OS-Linux-SNMP-Processcount</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>centreon_linux_snmp.pl</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>os::linux::snmp::plugin</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>processcount</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>$CENTREONPLUGINS$/centreon_linux_snmp.pl --plugin=os::linux::snmp::plugin --mode=processcount --hostname=$HOSTADDRESS$ --snmp-version='$_HOSTSNMPVERSION$' --snmp-community=******** --process-name='$_SERVICEPROCESSNAME$'</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>OS-Linux-SNMP-Traffic-Name</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>centreon_linux_snmp.pl</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>os::linux::snmp::plugin</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>interfaces</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>$CENTREONPLUGINS$/centreon_linux_snmp.pl --plugin=os::linux::snmp::plugin --mode=interfaces --hostname=$HOSTADDRESS$ --snmp-version='$_HOSTSNMPVERSION$' --snmp-community=******** --interface='$_SERVICEINTERFACENAME$' --name --add-traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>OS-Windows-NSClient-Services</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>check_nrpe</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>$USER1$/check_nrpe -H $HOSTADDRESS$ -p 5666 -c check_centreon_plugins -a 'os::windows::local::plugin' 'service' '--filter-name=$_SERVICESERVICENAME$'</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>OS-Windows-SNMP-Cpu</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>centreon_windows_snmp.pl</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>os::windows::snmp::plugin</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>2</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>$CENTREONPLUGINS$/centreon_windows_snmp.pl --plugin=os::windows::snmp::plugin --mode=cpu --hostname=$HOSTADDRESS$ --snmp-version='$_HOSTSNMPVERSION$' --snmp-community=********</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>OS-Windows-SNMP-Storage</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>centreon_windows_snmp.pl</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>os::windows::snmp::plugin</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>storage</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>$CENTREONPLUGINS$/centreon_windows_snmp.pl --plugin=os::windows::snmp::plugin --mode=storage --hostname=$HOSTADDRESS$ --snmp-version='$_HOSTSNMPVERSION$' --snmp-community=******** --storage='$_SERVICEDISKNAME$'</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G18"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="140" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Mode d'emploi de la matrice</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1. « Matrice templates services » : une ligne par template de service Centreon (et par commande pour les services sans template). C'est l'unité de décision principale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Lire la colonne « Proposition » (calculée), puis saisir la « Décision finale » (liste déroulante) et le « Template / item Zabbix cible ». Les cellules jaunes sont à remplir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2. « Matrice templates hôtes » : même principe pour les templates d'hôte → templates Zabbix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>3. « Services » : inventaire détaillé hôte par hôte. La colonne « Décision (template) » reprend automatiquement la décision du template ; « Décision (service) » permet une exception ponctuelle ; « Décision effective » donne le résultat final (filtrable).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>4. « Hôtes » : liste des hôtes avec interface et templates Zabbix suggérés, proxy = collecteur Centreon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>5. Onglets « Croisé » : vue matricielle hôtes × templates pour repérer les profils d'hôtes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Stratégies</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Natif : couvert par un template officiel Zabbix → effort faible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Adapter : équivalent Zabbix existant (clé d'item, check simple, LLD) à paramétrer → effort moyen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Développer : check spécifique (script maison) → UserParameter / script externe / plugin agent 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Abandonner : sans objet sous Zabbix (dummy, supervision de Centreon lui-même...).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Priorité : Haute / Moyenne / Basse selon le nombre d'hôtes concernés (seuils paramétrables).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Les correspondances proviennent de mapping/zabbix_mapping.yaml : adaptez-le puis régénérez la matrice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Les secrets détectés dans les lignes de commande (--password, community SNMP...) sont masqués.</t>
         </is>
       </c>
     </row>
@@ -1290,7 +2479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA23"/>
+  <dimension ref="A1:AB23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -1320,6 +2509,7 @@
     <col width="19" customWidth="1" min="25" max="25"/>
     <col width="32" customWidth="1" min="26" max="26"/>
     <col width="15" customWidth="1" min="27" max="27"/>
+    <col width="30" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1456,6 +2646,11 @@
       <c r="AA1" s="4" t="inlineStr">
         <is>
           <t>Commentaire</t>
+        </is>
+      </c>
+      <c r="AB1" s="4" t="inlineStr">
+        <is>
+          <t>Template Zabbix disponible</t>
         </is>
       </c>
     </row>
@@ -1559,6 +2754,11 @@
       <c r="Y2" s="5" t="inlineStr"/>
       <c r="Z2" s="5" t="inlineStr"/>
       <c r="AA2" s="5" t="inlineStr"/>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1672,6 +2872,11 @@
       <c r="Y3" s="5" t="inlineStr"/>
       <c r="Z3" s="5" t="inlineStr"/>
       <c r="AA3" s="5" t="inlineStr"/>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1785,6 +2990,11 @@
       <c r="Y4" s="5" t="inlineStr"/>
       <c r="Z4" s="5" t="inlineStr"/>
       <c r="AA4" s="5" t="inlineStr"/>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1898,6 +3108,11 @@
       <c r="Y5" s="5" t="inlineStr"/>
       <c r="Z5" s="5" t="inlineStr"/>
       <c r="AA5" s="5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2007,6 +3222,11 @@
       <c r="Y6" s="5" t="inlineStr"/>
       <c r="Z6" s="5" t="inlineStr"/>
       <c r="AA6" s="5" t="inlineStr"/>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2120,6 +3340,11 @@
       <c r="Y7" s="5" t="inlineStr"/>
       <c r="Z7" s="5" t="inlineStr"/>
       <c r="AA7" s="5" t="inlineStr"/>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2221,6 +3446,7 @@
       <c r="Y8" s="5" t="inlineStr"/>
       <c r="Z8" s="5" t="inlineStr"/>
       <c r="AA8" s="5" t="inlineStr"/>
+      <c r="AB8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2334,6 +3560,7 @@
       <c r="Y9" s="5" t="inlineStr"/>
       <c r="Z9" s="5" t="inlineStr"/>
       <c r="AA9" s="5" t="inlineStr"/>
+      <c r="AB9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2447,6 +3674,11 @@
       <c r="Y10" s="5" t="inlineStr"/>
       <c r="Z10" s="5" t="inlineStr"/>
       <c r="AA10" s="5" t="inlineStr"/>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2560,6 +3792,11 @@
       <c r="Y11" s="5" t="inlineStr"/>
       <c r="Z11" s="5" t="inlineStr"/>
       <c r="AA11" s="5" t="inlineStr"/>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2649,6 +3886,7 @@
       <c r="Y12" s="5" t="inlineStr"/>
       <c r="Z12" s="5" t="inlineStr"/>
       <c r="AA12" s="5" t="inlineStr"/>
+      <c r="AB12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2762,6 +4000,11 @@
       <c r="Y13" s="5" t="inlineStr"/>
       <c r="Z13" s="5" t="inlineStr"/>
       <c r="AA13" s="5" t="inlineStr"/>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2871,6 +4114,7 @@
       <c r="Y14" s="5" t="inlineStr"/>
       <c r="Z14" s="5" t="inlineStr"/>
       <c r="AA14" s="5" t="inlineStr"/>
+      <c r="AB14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2976,6 +4220,7 @@
       <c r="Y15" s="5" t="inlineStr"/>
       <c r="Z15" s="5" t="inlineStr"/>
       <c r="AA15" s="5" t="inlineStr"/>
+      <c r="AB15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3077,6 +4322,11 @@
       <c r="Y16" s="5" t="inlineStr"/>
       <c r="Z16" s="5" t="inlineStr"/>
       <c r="AA16" s="5" t="inlineStr"/>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3174,6 +4424,7 @@
       <c r="Y17" s="5" t="inlineStr"/>
       <c r="Z17" s="5" t="inlineStr"/>
       <c r="AA17" s="5" t="inlineStr"/>
+      <c r="AB17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3243,6 +4494,7 @@
       <c r="Y18" s="5" t="inlineStr"/>
       <c r="Z18" s="5" t="inlineStr"/>
       <c r="AA18" s="5" t="inlineStr"/>
+      <c r="AB18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3312,6 +4564,7 @@
       <c r="Y19" s="5" t="inlineStr"/>
       <c r="Z19" s="5" t="inlineStr"/>
       <c r="AA19" s="5" t="inlineStr"/>
+      <c r="AB19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3381,6 +4634,7 @@
       <c r="Y20" s="5" t="inlineStr"/>
       <c r="Z20" s="5" t="inlineStr"/>
       <c r="AA20" s="5" t="inlineStr"/>
+      <c r="AB20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3482,6 +4736,11 @@
       <c r="Y21" s="5" t="inlineStr"/>
       <c r="Z21" s="5" t="inlineStr"/>
       <c r="AA21" s="5" t="inlineStr"/>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3567,6 +4826,7 @@
       <c r="Y22" s="5" t="inlineStr"/>
       <c r="Z22" s="5" t="inlineStr"/>
       <c r="AA22" s="5" t="inlineStr"/>
+      <c r="AB22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3668,9 +4928,14 @@
       <c r="Y23" s="5" t="inlineStr"/>
       <c r="Z23" s="5" t="inlineStr"/>
       <c r="AA23" s="5" t="inlineStr"/>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AA23"/>
+  <autoFilter ref="A1:AB23"/>
   <conditionalFormatting sqref="X2:X23">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>X2="Migrer (template natif)"</formula>
@@ -3732,7 +4997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R13"/>
+  <dimension ref="A1:S13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -3753,6 +5018,7 @@
     <col width="19" customWidth="1" min="16" max="16"/>
     <col width="25" customWidth="1" min="17" max="17"/>
     <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="30" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -3846,6 +5112,11 @@
           <t>Commentaire</t>
         </is>
       </c>
+      <c r="S1" s="4" t="inlineStr">
+        <is>
+          <t>Template Zabbix disponible</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3920,6 +5191,11 @@
       <c r="P2" s="5" t="inlineStr"/>
       <c r="Q2" s="5" t="inlineStr"/>
       <c r="R2" s="5" t="inlineStr"/>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3990,6 +5266,11 @@
       <c r="P3" s="5" t="inlineStr"/>
       <c r="Q3" s="5" t="inlineStr"/>
       <c r="R3" s="5" t="inlineStr"/>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4064,6 +5345,11 @@
       <c r="P4" s="5" t="inlineStr"/>
       <c r="Q4" s="5" t="inlineStr"/>
       <c r="R4" s="5" t="inlineStr"/>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4138,6 +5424,11 @@
       <c r="P5" s="5" t="inlineStr"/>
       <c r="Q5" s="5" t="inlineStr"/>
       <c r="R5" s="5" t="inlineStr"/>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4208,6 +5499,11 @@
       <c r="P6" s="5" t="inlineStr"/>
       <c r="Q6" s="5" t="inlineStr"/>
       <c r="R6" s="5" t="inlineStr"/>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4270,6 +5566,7 @@
       <c r="P7" s="5" t="inlineStr"/>
       <c r="Q7" s="5" t="inlineStr"/>
       <c r="R7" s="5" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4340,6 +5637,11 @@
       <c r="P8" s="5" t="inlineStr"/>
       <c r="Q8" s="5" t="inlineStr"/>
       <c r="R8" s="5" t="inlineStr"/>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4410,6 +5712,11 @@
       <c r="P9" s="5" t="inlineStr"/>
       <c r="Q9" s="5" t="inlineStr"/>
       <c r="R9" s="5" t="inlineStr"/>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4480,6 +5787,11 @@
       <c r="P10" s="5" t="inlineStr"/>
       <c r="Q10" s="5" t="inlineStr"/>
       <c r="R10" s="5" t="inlineStr"/>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4550,6 +5862,11 @@
       <c r="P11" s="5" t="inlineStr"/>
       <c r="Q11" s="5" t="inlineStr"/>
       <c r="R11" s="5" t="inlineStr"/>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4616,6 +5933,11 @@
       <c r="P12" s="5" t="inlineStr"/>
       <c r="Q12" s="5" t="inlineStr"/>
       <c r="R12" s="5" t="inlineStr"/>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4686,9 +6008,14 @@
       <c r="P13" s="5" t="inlineStr"/>
       <c r="Q13" s="5" t="inlineStr"/>
       <c r="R13" s="5" t="inlineStr"/>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R13"/>
+  <autoFilter ref="A1:S13"/>
   <conditionalFormatting sqref="O2:O13">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>O2="Migrer (template natif)"</formula>
@@ -5575,7 +6902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V36"/>
+  <dimension ref="A1:X36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5596,10 +6923,12 @@
     <col width="45" customWidth="1" min="16" max="16"/>
     <col width="13" customWidth="1" min="17" max="17"/>
     <col width="25" customWidth="1" min="18" max="18"/>
-    <col width="23" customWidth="1" min="19" max="19"/>
+    <col width="25" customWidth="1" min="19" max="19"/>
     <col width="22" customWidth="1" min="20" max="20"/>
-    <col width="22" customWidth="1" min="21" max="21"/>
+    <col width="25" customWidth="1" min="21" max="21"/>
     <col width="15" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
+    <col width="23" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -5713,6 +7042,16 @@
           <t>Commentaire</t>
         </is>
       </c>
+      <c r="W1" s="4" t="inlineStr">
+        <is>
+          <t>Hôte dans Zabbix</t>
+        </is>
+      </c>
+      <c r="X1" s="4" t="inlineStr">
+        <is>
+          <t>Statut Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -5807,6 +7146,16 @@
         <v/>
       </c>
       <c r="V2" s="5" t="inlineStr"/>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Couvert dans Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5901,6 +7250,16 @@
         <v/>
       </c>
       <c r="V3" s="5" t="inlineStr"/>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>Couvert dans Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5995,6 +7354,16 @@
         <v/>
       </c>
       <c r="V4" s="5" t="inlineStr"/>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>Couvert dans Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -6089,6 +7458,16 @@
         <v/>
       </c>
       <c r="V5" s="5" t="inlineStr"/>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>Template à lier</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6179,6 +7558,16 @@
         <v/>
       </c>
       <c r="V6" s="5" t="inlineStr"/>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>Template à lier</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -6269,6 +7658,16 @@
         <v/>
       </c>
       <c r="V7" s="5" t="inlineStr"/>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>À créer dans Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -6355,6 +7754,16 @@
         <v/>
       </c>
       <c r="V8" s="5" t="inlineStr"/>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -6441,6 +7850,16 @@
         <v/>
       </c>
       <c r="V9" s="5" t="inlineStr"/>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6535,6 +7954,16 @@
         <v/>
       </c>
       <c r="V10" s="5" t="inlineStr"/>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6617,6 +8046,16 @@
         <v/>
       </c>
       <c r="V11" s="5" t="inlineStr"/>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6711,6 +8150,16 @@
         <v/>
       </c>
       <c r="V12" s="5" t="inlineStr"/>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6801,6 +8250,16 @@
         <v/>
       </c>
       <c r="V13" s="5" t="inlineStr"/>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6895,6 +8354,16 @@
         <v/>
       </c>
       <c r="V14" s="5" t="inlineStr"/>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>Couvert dans Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6989,6 +8458,16 @@
         <v/>
       </c>
       <c r="V15" s="5" t="inlineStr"/>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>Couvert dans Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -7083,6 +8562,16 @@
         <v/>
       </c>
       <c r="V16" s="5" t="inlineStr"/>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>Couvert dans Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -7181,6 +8670,16 @@
         <v/>
       </c>
       <c r="V17" s="5" t="inlineStr"/>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>Template à lier</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -7275,6 +8774,16 @@
         <v/>
       </c>
       <c r="V18" s="5" t="inlineStr"/>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>Couvert dans Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -7369,6 +8878,16 @@
         <v/>
       </c>
       <c r="V19" s="5" t="inlineStr"/>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>Non migré (décision)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -7459,6 +8978,16 @@
         <v/>
       </c>
       <c r="V20" s="5" t="inlineStr"/>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>Couvert dans Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -7553,6 +9082,16 @@
         <v/>
       </c>
       <c r="V21" s="5" t="inlineStr"/>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -7647,6 +9186,16 @@
         <v/>
       </c>
       <c r="V22" s="5" t="inlineStr"/>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -7741,6 +9290,16 @@
         <v/>
       </c>
       <c r="V23" s="5" t="inlineStr"/>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -7839,6 +9398,16 @@
         <v/>
       </c>
       <c r="V24" s="5" t="inlineStr"/>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -7933,6 +9502,16 @@
         <v/>
       </c>
       <c r="V25" s="5" t="inlineStr"/>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -8023,6 +9602,16 @@
         <v/>
       </c>
       <c r="V26" s="5" t="inlineStr"/>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -8117,6 +9706,16 @@
         <v/>
       </c>
       <c r="V27" s="5" t="inlineStr"/>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>Template à lier</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -8211,6 +9810,16 @@
         <v/>
       </c>
       <c r="V28" s="5" t="inlineStr"/>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>Template à lier</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -8297,6 +9906,16 @@
         <v/>
       </c>
       <c r="V29" s="5" t="inlineStr"/>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>Couvert dans Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -8391,6 +10010,16 @@
         <v/>
       </c>
       <c r="V30" s="5" t="inlineStr"/>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -8485,6 +10114,16 @@
         <v/>
       </c>
       <c r="V31" s="5" t="inlineStr"/>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -8567,6 +10206,16 @@
         <v/>
       </c>
       <c r="V32" s="5" t="inlineStr"/>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>Non migré (décision)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -8661,6 +10310,16 @@
         <v/>
       </c>
       <c r="V33" s="5" t="inlineStr"/>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>Non migré (décision)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -8755,6 +10414,16 @@
         <v/>
       </c>
       <c r="V34" s="5" t="inlineStr"/>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>À créer dans Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -8849,6 +10518,16 @@
         <v/>
       </c>
       <c r="V35" s="5" t="inlineStr"/>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>À créer dans Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -8935,9 +10614,19 @@
         <v/>
       </c>
       <c r="V36" s="5" t="inlineStr"/>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V36"/>
+  <autoFilter ref="A1:X36"/>
   <conditionalFormatting sqref="R2:R36">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>R2="Migrer (template natif)"</formula>
@@ -9030,6 +10719,38 @@
       <formula>U2="Migrer"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="X2:X36">
+    <cfRule type="expression" priority="29" dxfId="0">
+      <formula>X2="Présent – templates OK"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="30" dxfId="0">
+      <formula>X2="Couvert dans Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="31" dxfId="4">
+      <formula>X2="Présent – templates à lier"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="32" dxfId="4">
+      <formula>X2="Template à lier"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="33" dxfId="1">
+      <formula>X2="Présent"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="34" dxfId="6">
+      <formula>X2="Absent de Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="35" dxfId="6">
+      <formula>X2="Hôte absent de Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="36" dxfId="2">
+      <formula>X2="À créer dans Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="37" dxfId="3">
+      <formula>X2="Non migré (décision)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="38" dxfId="6">
+      <formula>X2="Non (à importer)"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="T2:T36" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Décision" error="Choisir une valeur dans la liste" type="list">
       <formula1>"Migrer (template natif),Migrer (adapter),Migrer (développer),Ne pas migrer,À analyser,Hérité (pas d'action directe)"</formula1>
@@ -9490,10 +11211,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B3:M11">
-    <cfRule type="expression" priority="1" dxfId="6">
+    <cfRule type="expression" priority="1" dxfId="7">
       <formula>B3="D"</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="7">
+    <cfRule type="expression" priority="2" dxfId="8">
       <formula>AND(B3&lt;&gt;"",B3&lt;&gt;"D")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9898,10 +11619,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B3:Q11">
-    <cfRule type="expression" priority="1" dxfId="6">
+    <cfRule type="expression" priority="1" dxfId="7">
       <formula>B3="D"</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="7">
+    <cfRule type="expression" priority="2" dxfId="8">
       <formula>AND(B3&lt;&gt;"",B3&lt;&gt;"D")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9915,612 +11636,718 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:Q10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="90" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="19" customWidth="1" min="13" max="13"/>
+    <col width="42" customWidth="1" min="14" max="14"/>
+    <col width="45" customWidth="1" min="15" max="15"/>
+    <col width="42" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Commande</t>
+          <t>Hôte Centreon</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Adresse</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>Exécutable</t>
+          <t>Collecteur Centreon</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Plugin</t>
+          <t>Actif Centreon</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>Mode</t>
+          <t>Statut Zabbix</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>Nb services</t>
+          <t>Correspondance</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
-          <t>Ligne de commande</t>
+          <t>Hôte Zabbix</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Nom visible Zabbix</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Activé dans Zabbix</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Proxy Zabbix</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Groupes Zabbix</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Interfaces Zabbix</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>Nb items Zabbix</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>Templates Zabbix liés</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>Templates Zabbix suggérés</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
+          <t>Templates à lier</t>
+        </is>
+      </c>
+      <c r="Q1" s="4" t="inlineStr">
+        <is>
+          <t>Nb services Centreon</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>App-DB-MySQL-Connections</t>
+          <t>srv-lnx-db01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>check</t>
+          <t>10.0.10.21</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>centreon_mysql.pl</t>
+          <t>Poller-DC1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>database::mysql::plugin</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>connection-time</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1</v>
+          <t>Présent – templates à lier</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Nom</t>
+        </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>$CENTREONPLUGINS$/centreon_mysql.pl --plugin=database::mysql::plugin --mode=connection-time --host=$HOSTADDRESS$ --username='$_HOSTMYSQLUSERNAME$' --password=********</t>
-        </is>
+          <t>srv-lnx-db01</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>srv-lnx-db01</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>proxy-dc1</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Linux servers</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>SNMP</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>120</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Linux by SNMP</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Linux by SNMP, MySQL by Zabbix agent 2, ICMP Ping</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>MySQL by Zabbix agent 2, ICMP Ping</t>
+        </is>
+      </c>
+      <c r="Q2" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>App-Monitoring-Centreon-Ping</t>
+          <t>srv-lnx-erp01</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>check</t>
+          <t>10.0.10.31</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>check_icmp</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="n">
-        <v>5</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>$USER1$/check_icmp -H $HOSTADDRESS$ -n $_SERVICEPACKETNUMBER$ -w $_SERVICEWARNING$ -c $_SERVICECRITICAL$</t>
-        </is>
+          <t>Poller-DC2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Absent de Zabbix</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Linux by SNMP, ICMP Ping</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Linux by SNMP, ICMP Ping</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>App-Protocol-HTTP-Response</t>
+          <t>srv-lnx-web01</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>check</t>
+          <t>10.0.10.11</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>centreon_protocol_http.pl</t>
+          <t>Poller-DC1</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>apps::protocols::http::plugin</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>response</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>2</v>
+          <t>Présent – templates OK</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Nom</t>
+        </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>$CENTREONPLUGINS$/centreon_protocol_http.pl --plugin=apps::protocols::http::plugin --mode=response --hostname=$_SERVICEURLHOST$ --urlpath='$_SERVICEURLPATH$' --ssl-opt='SSL_verify_mode =&gt; SSL_VERIFY_NONE'</t>
-        </is>
+          <t>srv-lnx-web01</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>srv-lnx-web01</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>proxy-dc1</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Linux servers, Web</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>SNMP</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>182</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Linux by SNMP, Apache by HTTP, ICMP Ping</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Linux by SNMP, Apache by HTTP, ICMP Ping</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>App-Webserver-Apache-Requests</t>
+          <t>srv-lnx-web02</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>check</t>
+          <t>10.0.10.12</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>centreon_apache_serverstatus.pl</t>
+          <t>Poller-DC1</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>apps::apache::serverstatus::plugin</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>requests</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>2</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>$CENTREONPLUGINS$/centreon_apache_serverstatus.pl --plugin=apps::apache::serverstatus::plugin --mode=requests --hostname=$HOSTADDRESS$</t>
-        </is>
+          <t>Absent de Zabbix</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Linux by SNMP, Apache by HTTP, ICMP Ping</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Linux by SNMP, Apache by HTTP, ICMP Ping</t>
+        </is>
+      </c>
+      <c r="Q5" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>base_host_alive</t>
+          <t>srv-win-ad01</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>check</t>
+          <t>10.0.20.11</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>check_icmp</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="n">
-        <v>0</v>
+          <t>Poller-DC1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Présent – templates à lier</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Nom</t>
+        </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>$USER1$/check_icmp -H $HOSTADDRESS$ -w 3000.0,80% -c 5000.0,100% -p 1</t>
-        </is>
+          <t>SRV-WIN-AD01</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>SRV-WIN-AD01</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>proxy-dc1</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Windows servers</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>240</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Windows by Zabbix agent</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Windows by SNMP, Windows by Zabbix agent</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Windows by SNMP</t>
+        </is>
+      </c>
+      <c r="Q6" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>check_centreon_dummy</t>
+          <t>srv-win-file01</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>check</t>
+          <t>10.0.20.12</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>check_dummy</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>$USER1$/check_dummy -o $ARG1$ -s $ARG2$</t>
-        </is>
+          <t>Poller-DC2</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Absent de Zabbix</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Windows by SNMP</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Windows by SNMP</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>check_erp_batch</t>
+          <t>sw-acc-02</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>check</t>
+          <t>10.0.0.2</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>check_erp_batch.sh</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="n">
-        <v>3</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>$USER2$/check_erp_batch.sh -H $HOSTADDRESS$ -j $ARG1$ -w $ARG2$ -c $ARG3$</t>
-        </is>
+          <t>Poller-DC2</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Absent de Zabbix</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Cisco IOS by SNMP</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Cisco IOS by SNMP</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Net-Cisco-Standard-SNMP-Environment</t>
+          <t>sw-core-01</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>check</t>
+          <t>10.0.0.1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>centreon_cisco_standard_snmp.pl</t>
+          <t>Poller-DC1</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>network::cisco::standard::snmp::plugin</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>environment</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
+          <t>Présent – templates OK</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Adresse IP</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>core-switch</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>core-switch</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>proxy-dc1</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Network</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>SNMP</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>640</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Cisco IOS by SNMP</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Cisco IOS by SNMP</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="n">
         <v>2</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>$CENTREONPLUGINS$/centreon_cisco_standard_snmp.pl --plugin=network::cisco::standard::snmp::plugin --mode=environment --hostname=$HOSTADDRESS$ --snmp-community=********</t>
-        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Net-Cisco-Standard-SNMP-Traffic-Name</t>
+          <t>ups-dc1</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>check</t>
+          <t>10.0.0.50</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>centreon_cisco_standard_snmp.pl</t>
+          <t>Poller-DC1</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>network::cisco::standard::snmp::plugin</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>interfaces</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
+          <t>Absent de Zabbix</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>APC UPS by SNMP, ICMP Ping</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>APC UPS by SNMP, ICMP Ping</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
         <v>1</v>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>$CENTREONPLUGINS$/centreon_cisco_standard_snmp.pl --plugin=network::cisco::standard::snmp::plugin --mode=interfaces --hostname=$HOSTADDRESS$ --snmp-community=******** --interface='$_SERVICEINTERFACENAME$' --name</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>OS-Linux-SNMP-Cpu</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>check</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>centreon_linux_snmp.pl</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>os::linux::snmp::plugin</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>cpu</t>
-        </is>
-      </c>
-      <c r="F11" t="n">
-        <v>4</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>$CENTREONPLUGINS$/centreon_linux_snmp.pl --plugin=os::linux::snmp::plugin --mode=cpu --hostname=$HOSTADDRESS$ --snmp-version='$_HOSTSNMPVERSION$' --snmp-community=******** --warning-average='$_SERVICEWARNING$' --critical-average='$_SERVICECRITICAL$'</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>OS-Linux-SNMP-Disk-Name</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>check</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>centreon_linux_snmp.pl</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>os::linux::snmp::plugin</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>storage</t>
-        </is>
-      </c>
-      <c r="F12" t="n">
-        <v>3</v>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>$CENTREONPLUGINS$/centreon_linux_snmp.pl --plugin=os::linux::snmp::plugin --mode=storage --hostname=$HOSTADDRESS$ --snmp-version='$_HOSTSNMPVERSION$' --snmp-community=******** --storage='$_SERVICEDISKNAME$' --name --warning-usage='$_SERVICEWARNING$' --critical-usage='$_SERVICECRITICAL$'</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>OS-Linux-SNMP-Memory</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>check</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>centreon_linux_snmp.pl</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>os::linux::snmp::plugin</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>memory</t>
-        </is>
-      </c>
-      <c r="F13" t="n">
-        <v>5</v>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>$CENTREONPLUGINS$/centreon_linux_snmp.pl --plugin=os::linux::snmp::plugin --mode=memory --hostname=$HOSTADDRESS$ --snmp-version='$_HOSTSNMPVERSION$' --snmp-community=******** --warning-usage='$_SERVICEWARNING$' --critical-usage='$_SERVICECRITICAL$'</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>OS-Linux-SNMP-Processcount</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>check</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>centreon_linux_snmp.pl</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>os::linux::snmp::plugin</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>processcount</t>
-        </is>
-      </c>
-      <c r="F14" t="n">
-        <v>1</v>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>$CENTREONPLUGINS$/centreon_linux_snmp.pl --plugin=os::linux::snmp::plugin --mode=processcount --hostname=$HOSTADDRESS$ --snmp-version='$_HOSTSNMPVERSION$' --snmp-community=******** --process-name='$_SERVICEPROCESSNAME$'</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>OS-Linux-SNMP-Traffic-Name</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>check</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>centreon_linux_snmp.pl</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>os::linux::snmp::plugin</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>interfaces</t>
-        </is>
-      </c>
-      <c r="F15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>$CENTREONPLUGINS$/centreon_linux_snmp.pl --plugin=os::linux::snmp::plugin --mode=interfaces --hostname=$HOSTADDRESS$ --snmp-version='$_HOSTSNMPVERSION$' --snmp-community=******** --interface='$_SERVICEINTERFACENAME$' --name --add-traffic</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>OS-Windows-NSClient-Services</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>check</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>check_nrpe</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>$USER1$/check_nrpe -H $HOSTADDRESS$ -p 5666 -c check_centreon_plugins -a 'os::windows::local::plugin' 'service' '--filter-name=$_SERVICESERVICENAME$'</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>OS-Windows-SNMP-Cpu</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>check</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>centreon_windows_snmp.pl</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>os::windows::snmp::plugin</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>cpu</t>
-        </is>
-      </c>
-      <c r="F17" t="n">
-        <v>2</v>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>$CENTREONPLUGINS$/centreon_windows_snmp.pl --plugin=os::windows::snmp::plugin --mode=cpu --hostname=$HOSTADDRESS$ --snmp-version='$_HOSTSNMPVERSION$' --snmp-community=********</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>OS-Windows-SNMP-Storage</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>check</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>centreon_windows_snmp.pl</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>os::windows::snmp::plugin</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>storage</t>
-        </is>
-      </c>
-      <c r="F18" t="n">
-        <v>2</v>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>$CENTREONPLUGINS$/centreon_windows_snmp.pl --plugin=os::windows::snmp::plugin --mode=storage --hostname=$HOSTADDRESS$ --snmp-version='$_HOSTSNMPVERSION$' --snmp-community=******** --storage='$_SERVICEDISKNAME$'</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G18"/>
+  <autoFilter ref="A1:Q10"/>
+  <conditionalFormatting sqref="E2:E10">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>E2="Présent – templates OK"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>E2="Couvert dans Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="4">
+      <formula>E2="Présent – templates à lier"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="4">
+      <formula>E2="Template à lier"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="1">
+      <formula>E2="Présent"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="6">
+      <formula>E2="Absent de Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" dxfId="6">
+      <formula>E2="Hôte absent de Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="2">
+      <formula>E2="À créer dans Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="9" dxfId="3">
+      <formula>E2="Non migré (décision)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="6">
+      <formula>E2="Non (à importer)"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10531,127 +12358,103 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="140" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>Mode d'emploi de la matrice</t>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Hôte Zabbix</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Nom visible</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Activé</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Adresses</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Proxy</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Groupes</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Templates liés</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Nb items</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1. « Matrice templates services » : une ligne par template de service Centreon (et par commande pour les services sans template). C'est l'unité de décision principale.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Lire la colonne « Proposition » (calculée), puis saisir la « Décision finale » (liste déroulante) et le « Template / item Zabbix cible ». Les cellules jaunes sont à remplir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2. « Matrice templates hôtes » : même principe pour les templates d'hôte → templates Zabbix.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>3. « Services » : inventaire détaillé hôte par hôte. La colonne « Décision (template) » reprend automatiquement la décision du template ; « Décision (service) » permet une exception ponctuelle ; « Décision effective » donne le résultat final (filtrable).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>4. « Hôtes » : liste des hôtes avec interface et templates Zabbix suggérés, proxy = collecteur Centreon.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>5. Onglets « Croisé » : vue matricielle hôtes × templates pour repérer les profils d'hôtes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>Stratégies</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Natif : couvert par un template officiel Zabbix → effort faible.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Adapter : équivalent Zabbix existant (clé d'item, check simple, LLD) à paramétrer → effort moyen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Développer : check spécifique (script maison) → UserParameter / script externe / plugin agent 2.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Abandonner : sans objet sous Zabbix (dummy, supervision de Centreon lui-même...).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Priorité : Haute / Moyenne / Basse selon le nombre d'hôtes concernés (seuils paramétrables).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Les correspondances proviennent de mapping/zabbix_mapping.yaml : adaptez-le puis régénérez la matrice.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Les secrets détectés dans les lignes de commande (--password, community SNMP...) sont masqués.</t>
-        </is>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>srv-lnx-new01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>srv-lnx-new01</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>10.0.10.99</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>proxy-dc1</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Linux servers</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Linux by Zabbix agent</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>95</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:H2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Hôte non migré => services non migrés, décisions groupées, corrélation services ↔ items Zabbix
- Un hôte en « Ne pas migrer » emporte tous ses services (colonne
  Décision (hôte), interface et formules Excel).
- Sélection multiple dans les tableaux modifiables (page, ou tous les
  résultats filtrés) et application groupée d'une valeur.
- Inventaire Zabbix : items et prototypes LLD des templates, templates
  liés. Corrélation par catégorie (règles « correlation » du mapping) :
  couvert par un item standard / template à importer / item à ajouter /
  spécificité à créer, approche recommandée, apport du standard.
- Nouvel onglet et feuille « Corrélation items Zabbix ».

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ss1AXzb7kQY6cySve132CB
</commit_message>
<xml_diff>
--- a/examples/matrice_exemple.xlsx
+++ b/examples/matrice_exemple.xlsx
@@ -17,18 +17,20 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparatif Zabbix hôtes" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Uniquement dans Zabbix" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Templates Zabbix" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commandes" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corrélation items Zabbix" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commandes" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Matrice templates services'!$A$1:$AB$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Matrice templates services'!$A$1:$AC$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matrice templates hôtes'!$A$1:$S$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Hôtes'!$A$1:$Q$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Services'!$A$1:$X$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Services'!$A$1:$AA$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Comparatif Zabbix hôtes'!$A$1:$Q$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Uniquement dans Zabbix'!$A$1:$H$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Templates Zabbix'!$A$1:$E$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Commandes'!$A$1:$G$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Templates Zabbix'!$A$1:$I$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Corrélation items Zabbix'!$A$1:$K$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Commandes'!$A$1:$G$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -546,7 +548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E74"/>
+  <dimension ref="A1:E80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -566,7 +568,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Généré le 15/10/2026 14:45</t>
+          <t>Généré le 15/10/2026 20:11</t>
         </is>
       </c>
     </row>
@@ -955,7 +957,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="44"/>
@@ -1074,208 +1076,127 @@
         <v>3</v>
       </c>
     </row>
+    <row r="57"/>
     <row r="58">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t>Top 15 des templates de service (par nombre de services)</t>
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Services Centreon : couverture par le standard Zabbix</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Nb services</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>Template de service</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
-        <is>
-          <t>Nb services</t>
-        </is>
-      </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>Nb hôtes</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
-          <t>Proposition</t>
-        </is>
-      </c>
-      <c r="E59" s="2" t="inlineStr">
-        <is>
-          <t>Template Zabbix suggéré</t>
-        </is>
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Base-Ping-LAN</t>
+          <t>Template standard à importer dans Zabbix</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>5</v>
-      </c>
-      <c r="C60" t="n">
-        <v>5</v>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>Migrer (template natif)</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>ICMP Ping</t>
-        </is>
+        <v>2</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>OS-Linux-Memory-SNMP-custom</t>
+          <t>Spécificité à créer</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>5</v>
-      </c>
-      <c r="C61" t="n">
         <v>4</v>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>Migrer (template natif)</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>Linux by SNMP</t>
-        </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>OS-Linux-Cpu-SNMP-custom</t>
+          <t>Non migré</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>4</v>
-      </c>
-      <c r="C62" t="n">
-        <v>4</v>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>Migrer (template natif)</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>Linux by SNMP</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>OS-Linux-Disk-Generic-Name-SNMP-custom</t>
-        </is>
-      </c>
-      <c r="B63" t="n">
         <v>3</v>
       </c>
-      <c r="C63" t="n">
-        <v>3</v>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>Migrer (template natif)</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>Linux by SNMP</t>
-        </is>
-      </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>App-Protocol-HTTP-Response-Time-custom</t>
-        </is>
-      </c>
-      <c r="B64" t="n">
-        <v>2</v>
-      </c>
-      <c r="C64" t="n">
-        <v>2</v>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>Migrer (adapter)</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Website by Browser</t>
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>Top 15 des templates de service (par nombre de services)</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>App-Webserver-Apache-Requests-custom</t>
-        </is>
-      </c>
-      <c r="B65" t="n">
-        <v>2</v>
-      </c>
-      <c r="C65" t="n">
-        <v>2</v>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>Migrer (template natif)</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>Apache by HTTP</t>
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Template de service</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Nb services</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Nb hôtes</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Proposition</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Template Zabbix suggéré</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ERP-Batch-Nocturne</t>
+          <t>Base-Ping-LAN</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C66" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>À analyser</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr"/>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ICMP Ping</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Net-Cisco-Standard-Environment-SNMP-custom</t>
+          <t>OS-Linux-Memory-SNMP-custom</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C67" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -1284,21 +1205,21 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>(template constructeur SNMP)</t>
+          <t>Linux by SNMP</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>OS-Windows-Cpu-SNMP-custom</t>
+          <t>OS-Linux-Cpu-SNMP-custom</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C68" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -1307,21 +1228,21 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Windows by SNMP</t>
+          <t>Linux by SNMP</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>OS-Windows-Disk-Generic-Name-SNMP-custom</t>
+          <t>OS-Linux-Disk-Generic-Name-SNMP-custom</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C69" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -1330,40 +1251,44 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Windows by SNMP</t>
+          <t>Linux by SNMP</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>(aucun template) check_erp_batch</t>
+          <t>App-Protocol-HTTP-Response-Time-custom</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C70" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>À analyser</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr"/>
+          <t>Migrer (adapter)</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Website by Browser</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>App-DB-MySQL-Connection-Time-custom</t>
+          <t>App-Webserver-Apache-Requests-custom</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C71" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -1372,70 +1297,200 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>MySQL by Zabbix agent 2</t>
+          <t>Apache by HTTP</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Net-Cisco-Standard-Traffic-Generic-Name-SNMP-custom</t>
+          <t>ERP-Batch-Nocturne</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C72" t="n">
         <v>1</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Migrer (template natif)</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>(template constructeur SNMP)</t>
-        </is>
-      </c>
+          <t>À analyser</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>OS-Linux-Process-Generic-SNMP-custom</t>
+          <t>Net-Cisco-Standard-Environment-SNMP-custom</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Migrer (adapter)</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr"/>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>(template constructeur SNMP)</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
+          <t>OS-Windows-Cpu-SNMP-custom</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>2</v>
+      </c>
+      <c r="C74" t="n">
+        <v>2</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Windows by SNMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>OS-Windows-Disk-Generic-Name-SNMP-custom</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>2</v>
+      </c>
+      <c r="C75" t="n">
+        <v>2</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Windows by SNMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>(aucun template) check_erp_batch</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>1</v>
+      </c>
+      <c r="C76" t="n">
+        <v>1</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>À analyser</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>App-DB-MySQL-Connection-Time-custom</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>1</v>
+      </c>
+      <c r="C77" t="n">
+        <v>1</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>MySQL by Zabbix agent 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Net-Cisco-Standard-Traffic-Generic-Name-SNMP-custom</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>1</v>
+      </c>
+      <c r="C78" t="n">
+        <v>1</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>(template constructeur SNMP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>OS-Linux-Process-Generic-SNMP-custom</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>1</v>
+      </c>
+      <c r="C79" t="n">
+        <v>1</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Migrer (adapter)</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
           <t>OS-Windows-Services-NRPE-custom</t>
         </is>
       </c>
-      <c r="B74" t="n">
+      <c r="B80" t="n">
         <v>1</v>
       </c>
-      <c r="C74" t="n">
+      <c r="C80" t="n">
         <v>1</v>
       </c>
-      <c r="D74" t="inlineStr">
+      <c r="D80" t="inlineStr">
         <is>
           <t>Migrer (template natif)</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr">
+      <c r="E80" t="inlineStr">
         <is>
           <t>Windows by Zabbix agent</t>
         </is>
@@ -1452,7 +1507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -1460,6 +1515,10 @@
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="33" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1488,6 +1547,26 @@
           <t>Utilisations Centreon (hôtes)</t>
         </is>
       </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Nb items</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Nb prototypes LLD</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Items correspondant à des services Centreon</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Apport du standard (sans équivalent Centreon)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1511,6 +1590,18 @@
       <c r="E2" t="n">
         <v>15</v>
       </c>
+      <c r="F2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I2" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1534,6 +1625,18 @@
       <c r="E3" t="n">
         <v>6</v>
       </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1557,6 +1660,18 @@
       <c r="E4" t="n">
         <v>5</v>
       </c>
+      <c r="F4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1580,6 +1695,18 @@
       <c r="E5" t="n">
         <v>4</v>
       </c>
+      <c r="F5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1603,6 +1730,18 @@
       <c r="E6" t="n">
         <v>2</v>
       </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1625,6 +1764,18 @@
       </c>
       <c r="E7" t="n">
         <v>2</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -1645,6 +1796,16 @@
       <c r="E8" t="n">
         <v>2</v>
       </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1667,6 +1828,18 @@
       </c>
       <c r="E9" t="n">
         <v>2</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -1687,9 +1860,19 @@
       <c r="E10" t="n">
         <v>1</v>
       </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E10"/>
+  <autoFilter ref="A1:I10"/>
   <conditionalFormatting sqref="B2:B10">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>B2="Présent – templates OK"</formula>
@@ -1720,6 +1903,21 @@
     </cfRule>
     <cfRule type="expression" priority="10" dxfId="6">
       <formula>B2="Non (à importer)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="11" dxfId="0">
+      <formula>B2="Couvert par un item standard"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="12" dxfId="4">
+      <formula>B2="Template standard sans item correspondant"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="13" dxfId="1">
+      <formula>B2="Template standard à importer dans Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" dxfId="2">
+      <formula>B2="Spécificité à créer"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="15" dxfId="3">
+      <formula>B2="Non migré"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1727,6 +1925,890 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="45" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Template de service</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Catégorie</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Plugin / mode</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Nb services</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Nb hôtes</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Template Zabbix examiné</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Items Zabbix correspondants</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Couverture standard</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Approche recommandée</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Item à créer (si spécifique)</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Décision</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Base-Ping-LAN</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Disponibilité</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>ICMP Ping</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>ICMP ping [icmpping] ; ICMP loss [icmppingloss] ; ICMP response time [icmppingsec]</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Standard : lier « ICMP Ping » (item « ICMP ping »)</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>OS-Linux-Memory-SNMP-custom</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Mémoire</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>os::linux::snmp::plugin / memory</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Linux by SNMP</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Memory utilization [vm.memory.util[snmp.vm.memory.util]]</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Standard : lier « Linux by SNMP » (item « Memory utilization »)</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>OS-Linux-Cpu-SNMP-custom</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>os::linux::snmp::plugin / cpu</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Linux by SNMP</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>CPU utilization [system.cpu.util[snmp.cpu.util]]</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Standard : lier « Linux by SNMP » (item « CPU utilization »)</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>OS-Linux-Disk-Generic-Name-SNMP-custom</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Disque</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>os::linux::snmp::plugin / storage</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Linux by SNMP</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>{#FSNAME}: Space utilization [vfs.fs.pused[storageUsedPercentage.{#SNMPINDEX}]] (LLD)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Standard : lier « Linux by SNMP » (item « {#FSNAME}: Space utilization »)</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>App-Webserver-Apache-Requests-custom</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>apps::apache::serverstatus::plugin / requests</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Apache by HTTP</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Requests per second [apache.requests.rate] ; Workers busy [apache.workers.busy]</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Standard : lier « Apache by HTTP » (item « Requests per second »)</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Net-Cisco-Standard-Environment-SNMP-custom</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Matériel</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>network::cisco::standard::snmp::plugin / environment</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Cisco IOS by SNMP</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>{#SENSOR_INFO}: Temperature [sensor.temp.value[ciscoEnvMonTemperatureValue.{#SNMPINDEX}]] (LLD)</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Standard : lier « Cisco IOS by SNMP » (item « {#SENSOR_INFO}: Temperature »)</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>OS-Windows-Cpu-SNMP-custom</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>os::windows::snmp::plugin / cpu</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Windows by SNMP</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>CPU utilization [system.cpu.util[snmp.cpu.util]]</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Standard : lier « Windows by SNMP » (item « CPU utilization »)</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>OS-Windows-Disk-Generic-Name-SNMP-custom</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Disque</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>os::windows::snmp::plugin / storage</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Windows by SNMP</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>{#FSNAME}: Space utilization [vfs.fs.pused[storageUsedPercentage.{#SNMPINDEX}]] (LLD)</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Standard : lier « Windows by SNMP » (item « {#FSNAME}: Space utilization »)</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>App-DB-MySQL-Connection-Time-custom</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Base de données</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>database::mysql::plugin / connection-time</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>MySQL by Zabbix agent 2</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Status [mysql.ping["{$MYSQL.DSN}"]] ; Connections per second [mysql.connections.rate]</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Standard : lier « MySQL by Zabbix agent 2 » (item « Status »)</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Net-Cisco-Standard-Traffic-Generic-Name-SNMP-custom</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Réseau</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>network::cisco::standard::snmp::plugin / interfaces</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Cisco IOS by SNMP</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Interface {#IFNAME}: Bits received [net.if.in[ifHCInOctets.{#SNMPINDEX}]] (LLD)</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Standard : lier « Cisco IOS by SNMP » (item « Interface {#IFNAME}: Bits received »)</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>OS-Windows-Services-NRPE-custom</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Services Windows</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Windows by Zabbix agent</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>State of service "{#SERVICE.NAME}" [service.info["{#SERVICE.NAME}",state]] (LLD)</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Standard : lier « Windows by Zabbix agent » (item « State of service "{#SERVICE.NAME}" »)</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Migrer (template natif)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>App-Protocol-HTTP-Response-Time-custom</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>apps::protocols::http::plugin / response</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Website by Browser</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Template standard à importer dans Zabbix</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Standard : importer puis lier « Website by Browser »</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Migrer (adapter)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ERP-Batch-Nocturne</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Spécifique</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Linux by SNMP, ICMP Ping</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Spécificité à créer</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Spécificité : créer UserParameter / script externe / plugin agent 2</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>UserParameter / script externe / plugin agent 2</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>À analyser</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>(aucun template) check_erp_batch</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Spécifique</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Linux by SNMP, ICMP Ping</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Spécificité à créer</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Spécificité : créer UserParameter / script externe / plugin agent 2</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>UserParameter / script externe / plugin agent 2</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>À analyser</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>OS-Linux-Process-Generic-SNMP-custom</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Processus</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>os::linux::snmp::plugin / processcount</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Linux by SNMP, MySQL by Zabbix agent 2, ICMP Ping</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Spécificité à créer</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Spécificité : créer Item SNMP hrSWRunName (à créer)</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Item SNMP hrSWRunName (à créer)</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Migrer (adapter)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Passive-Trap-Dummy</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Passif / Dummy</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Windows by SNMP</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Non migré</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Ne pas migrer</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:K17"/>
+  <conditionalFormatting sqref="H2:H17">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>H2="Présent – templates OK"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>H2="Couvert dans Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="4">
+      <formula>H2="Présent – templates à lier"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="4">
+      <formula>H2="Template à lier"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="1">
+      <formula>H2="Présent"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="6">
+      <formula>H2="Absent de Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" dxfId="6">
+      <formula>H2="Hôte absent de Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="2">
+      <formula>H2="À créer dans Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="9" dxfId="3">
+      <formula>H2="Non migré (décision)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="6">
+      <formula>H2="Non (à importer)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="11" dxfId="0">
+      <formula>H2="Couvert par un item standard"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="12" dxfId="4">
+      <formula>H2="Template standard sans item correspondant"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="13" dxfId="1">
+      <formula>H2="Template standard à importer dans Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" dxfId="2">
+      <formula>H2="Spécificité à créer"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="15" dxfId="3">
+      <formula>H2="Non migré"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2342,13 +3424,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -2407,62 +3489,69 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>6. « Corrélation items Zabbix » : pour chaque template de service Centreon, item(s) des templates Zabbix standards qui couvrent déjà la mesure, ou spécificité à créer. Démarche conseillée : lier d'abord les templates standards, puis n'ajouter que les spécificités.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Stratégies</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Natif : couvert par un template officiel Zabbix → effort faible.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Adapter : équivalent Zabbix existant (clé d'item, check simple, LLD) à paramétrer → effort moyen.</t>
+          <t>Natif : couvert par un template officiel Zabbix → effort faible.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Développer : check spécifique (script maison) → UserParameter / script externe / plugin agent 2.</t>
+          <t>Adapter : équivalent Zabbix existant (clé d'item, check simple, LLD) à paramétrer → effort moyen.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>Développer : check spécifique (script maison) → UserParameter / script externe / plugin agent 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>Abandonner : sans objet sous Zabbix (dummy, supervision de Centreon lui-même...).</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-    </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Priorité : Haute / Moyenne / Basse selon le nombre d'hôtes concernés (seuils paramétrables).</t>
-        </is>
-      </c>
+      <c r="A16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Les correspondances proviennent de mapping/zabbix_mapping.yaml : adaptez-le puis régénérez la matrice.</t>
+          <t>Priorité : Haute / Moyenne / Basse selon le nombre d'hôtes concernés (seuils paramétrables).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
+        <is>
+          <t>Les correspondances proviennent de mapping/zabbix_mapping.yaml : adaptez-le puis régénérez la matrice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Les secrets détectés dans les lignes de commande (--password, community SNMP...) sont masqués.</t>
         </is>
@@ -2479,7 +3568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB23"/>
+  <dimension ref="A1:AC23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -2510,6 +3599,7 @@
     <col width="32" customWidth="1" min="26" max="26"/>
     <col width="15" customWidth="1" min="27" max="27"/>
     <col width="30" customWidth="1" min="28" max="28"/>
+    <col width="42" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -2651,6 +3741,11 @@
       <c r="AB1" s="4" t="inlineStr">
         <is>
           <t>Template Zabbix disponible</t>
+        </is>
+      </c>
+      <c r="AC1" s="4" t="inlineStr">
+        <is>
+          <t>Couverture standard</t>
         </is>
       </c>
     </row>
@@ -2759,6 +3854,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2877,6 +3977,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2995,6 +4100,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3113,6 +4223,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3227,6 +4342,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>Template standard à importer dans Zabbix</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3345,6 +4465,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3447,6 +4572,11 @@
       <c r="Z8" s="5" t="inlineStr"/>
       <c r="AA8" s="5" t="inlineStr"/>
       <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>Spécificité à créer</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3561,6 +4691,11 @@
       <c r="Z9" s="5" t="inlineStr"/>
       <c r="AA9" s="5" t="inlineStr"/>
       <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3679,6 +4814,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3795,6 +4935,11 @@
       <c r="AB11" t="inlineStr">
         <is>
           <t>Oui</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -3887,6 +5032,11 @@
       <c r="Z12" s="5" t="inlineStr"/>
       <c r="AA12" s="5" t="inlineStr"/>
       <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>Spécificité à créer</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4005,6 +5155,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4115,6 +5270,11 @@
       <c r="Z14" s="5" t="inlineStr"/>
       <c r="AA14" s="5" t="inlineStr"/>
       <c r="AB14" t="inlineStr"/>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4221,6 +5381,11 @@
       <c r="Z15" s="5" t="inlineStr"/>
       <c r="AA15" s="5" t="inlineStr"/>
       <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>Spécificité à créer</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4327,6 +5492,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4425,6 +5595,11 @@
       <c r="Z17" s="5" t="inlineStr"/>
       <c r="AA17" s="5" t="inlineStr"/>
       <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>Non migré</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4495,6 +5670,7 @@
       <c r="Z18" s="5" t="inlineStr"/>
       <c r="AA18" s="5" t="inlineStr"/>
       <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4565,6 +5741,7 @@
       <c r="Z19" s="5" t="inlineStr"/>
       <c r="AA19" s="5" t="inlineStr"/>
       <c r="AB19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4635,6 +5812,7 @@
       <c r="Z20" s="5" t="inlineStr"/>
       <c r="AA20" s="5" t="inlineStr"/>
       <c r="AB20" t="inlineStr"/>
+      <c r="AC20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4741,6 +5919,7 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="AC21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4827,6 +6006,7 @@
       <c r="Z22" s="5" t="inlineStr"/>
       <c r="AA22" s="5" t="inlineStr"/>
       <c r="AB22" t="inlineStr"/>
+      <c r="AC22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4933,9 +6113,10 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="AC23" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AB23"/>
+  <autoFilter ref="A1:AC23"/>
   <conditionalFormatting sqref="X2:X23">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>X2="Migrer (template natif)"</formula>
@@ -4980,6 +6161,53 @@
     </cfRule>
     <cfRule type="expression" priority="14" dxfId="0">
       <formula>Y2="Migrer"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AC2:AC23">
+    <cfRule type="expression" priority="15" dxfId="0">
+      <formula>AC2="Présent – templates OK"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="16" dxfId="0">
+      <formula>AC2="Couvert dans Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="17" dxfId="4">
+      <formula>AC2="Présent – templates à lier"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="18" dxfId="4">
+      <formula>AC2="Template à lier"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="19" dxfId="1">
+      <formula>AC2="Présent"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="20" dxfId="6">
+      <formula>AC2="Absent de Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="21" dxfId="6">
+      <formula>AC2="Hôte absent de Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="22" dxfId="2">
+      <formula>AC2="À créer dans Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="23" dxfId="3">
+      <formula>AC2="Non migré (décision)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="24" dxfId="6">
+      <formula>AC2="Non (à importer)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="25" dxfId="0">
+      <formula>AC2="Couvert par un item standard"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="26" dxfId="4">
+      <formula>AC2="Template standard sans item correspondant"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="27" dxfId="1">
+      <formula>AC2="Template standard à importer dans Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="28" dxfId="2">
+      <formula>AC2="Spécificité à créer"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="29" dxfId="3">
+      <formula>AC2="Non migré"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -6902,7 +8130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X36"/>
+  <dimension ref="A1:AA36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6924,11 +8152,14 @@
     <col width="13" customWidth="1" min="17" max="17"/>
     <col width="25" customWidth="1" min="18" max="18"/>
     <col width="25" customWidth="1" min="19" max="19"/>
-    <col width="22" customWidth="1" min="20" max="20"/>
-    <col width="25" customWidth="1" min="21" max="21"/>
-    <col width="15" customWidth="1" min="22" max="22"/>
-    <col width="20" customWidth="1" min="23" max="23"/>
-    <col width="23" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="20" max="20"/>
+    <col width="22" customWidth="1" min="21" max="21"/>
+    <col width="25" customWidth="1" min="22" max="22"/>
+    <col width="15" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="23" customWidth="1" min="25" max="25"/>
+    <col width="45" customWidth="1" min="26" max="26"/>
+    <col width="42" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -7029,27 +8260,42 @@
       </c>
       <c r="T1" s="4" t="inlineStr">
         <is>
+          <t>Décision (hôte)</t>
+        </is>
+      </c>
+      <c r="U1" s="4" t="inlineStr">
+        <is>
           <t>Décision (service)</t>
         </is>
       </c>
-      <c r="U1" s="4" t="inlineStr">
+      <c r="V1" s="4" t="inlineStr">
         <is>
           <t>Décision effective</t>
         </is>
       </c>
-      <c r="V1" s="4" t="inlineStr">
+      <c r="W1" s="4" t="inlineStr">
         <is>
           <t>Commentaire</t>
         </is>
       </c>
-      <c r="W1" s="4" t="inlineStr">
+      <c r="X1" s="4" t="inlineStr">
         <is>
           <t>Hôte dans Zabbix</t>
         </is>
       </c>
-      <c r="X1" s="4" t="inlineStr">
+      <c r="Y1" s="4" t="inlineStr">
         <is>
           <t>Statut Zabbix</t>
+        </is>
+      </c>
+      <c r="Z1" s="4" t="inlineStr">
+        <is>
+          <t>Item Zabbix standard</t>
+        </is>
+      </c>
+      <c r="AA1" s="4" t="inlineStr">
+        <is>
+          <t>Couverture standard</t>
         </is>
       </c>
     </row>
@@ -7140,20 +8386,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G2,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G2,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G2,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T2" s="5" t="inlineStr"/>
-      <c r="U2">
-        <f>IF(T2&lt;&gt;"",T2,IF(E2="Non","Ne pas migrer",S2))</f>
+      <c r="T2">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A2,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A2,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A2,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V2" s="5" t="inlineStr"/>
-      <c r="W2" t="inlineStr">
+      <c r="U2" s="5" t="inlineStr"/>
+      <c r="V2">
+        <f>IF(T2="Ne pas migrer","Ne pas migrer",IF(U2&lt;&gt;"",U2,IF(E2="Non","Ne pas migrer",S2)))</f>
+        <v/>
+      </c>
+      <c r="W2" s="5" t="inlineStr"/>
+      <c r="X2" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t>Couvert dans Zabbix</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>CPU utilization [system.cpu.util[snmp.cpu.util]]</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -7244,20 +8504,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G3,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G3,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G3,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T3" s="5" t="inlineStr"/>
-      <c r="U3">
-        <f>IF(T3&lt;&gt;"",T3,IF(E3="Non","Ne pas migrer",S3))</f>
+      <c r="T3">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A3,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A3,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A3,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V3" s="5" t="inlineStr"/>
-      <c r="W3" t="inlineStr">
+      <c r="U3" s="5" t="inlineStr"/>
+      <c r="V3">
+        <f>IF(T3="Ne pas migrer","Ne pas migrer",IF(U3&lt;&gt;"",U3,IF(E3="Non","Ne pas migrer",S3)))</f>
+        <v/>
+      </c>
+      <c r="W3" s="5" t="inlineStr"/>
+      <c r="X3" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="Y3" t="inlineStr">
         <is>
           <t>Couvert dans Zabbix</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>{#FSNAME}: Space utilization [vfs.fs.pused[storageUsedPercentage.{#SNMPINDEX}]] (LLD)</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -7348,20 +8622,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G4,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G4,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G4,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T4" s="5" t="inlineStr"/>
-      <c r="U4">
-        <f>IF(T4&lt;&gt;"",T4,IF(E4="Non","Ne pas migrer",S4))</f>
+      <c r="T4">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A4,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A4,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A4,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V4" s="5" t="inlineStr"/>
-      <c r="W4" t="inlineStr">
+      <c r="U4" s="5" t="inlineStr"/>
+      <c r="V4">
+        <f>IF(T4="Ne pas migrer","Ne pas migrer",IF(U4&lt;&gt;"",U4,IF(E4="Non","Ne pas migrer",S4)))</f>
+        <v/>
+      </c>
+      <c r="W4" s="5" t="inlineStr"/>
+      <c r="X4" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>Couvert dans Zabbix</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>Memory utilization [vm.memory.util[snmp.vm.memory.util]]</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -7452,20 +8740,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G5,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G5,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G5,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T5" s="5" t="inlineStr"/>
-      <c r="U5">
-        <f>IF(T5&lt;&gt;"",T5,IF(E5="Non","Ne pas migrer",S5))</f>
+      <c r="T5">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A5,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A5,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A5,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V5" s="5" t="inlineStr"/>
-      <c r="W5" t="inlineStr">
+      <c r="U5" s="5" t="inlineStr"/>
+      <c r="V5">
+        <f>IF(T5="Ne pas migrer","Ne pas migrer",IF(U5&lt;&gt;"",U5,IF(E5="Non","Ne pas migrer",S5)))</f>
+        <v/>
+      </c>
+      <c r="W5" s="5" t="inlineStr"/>
+      <c r="X5" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr">
+      <c r="Y5" t="inlineStr">
         <is>
           <t>Template à lier</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>Status [mysql.ping["{$MYSQL.DSN}"]] … (+1)</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -7552,20 +8854,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G6,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G6,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G6,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T6" s="5" t="inlineStr"/>
-      <c r="U6">
-        <f>IF(T6&lt;&gt;"",T6,IF(E6="Non","Ne pas migrer",S6))</f>
+      <c r="T6">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A6,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A6,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A6,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V6" s="5" t="inlineStr"/>
-      <c r="W6" t="inlineStr">
+      <c r="U6" s="5" t="inlineStr"/>
+      <c r="V6">
+        <f>IF(T6="Ne pas migrer","Ne pas migrer",IF(U6&lt;&gt;"",U6,IF(E6="Non","Ne pas migrer",S6)))</f>
+        <v/>
+      </c>
+      <c r="W6" s="5" t="inlineStr"/>
+      <c r="X6" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr">
+      <c r="Y6" t="inlineStr">
         <is>
           <t>Template à lier</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>ICMP ping [icmpping] … (+2)</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -7652,20 +8968,30 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G7,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G7,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G7,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T7" s="5" t="inlineStr"/>
-      <c r="U7">
-        <f>IF(T7&lt;&gt;"",T7,IF(E7="Non","Ne pas migrer",S7))</f>
+      <c r="T7">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A7,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A7,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A7,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V7" s="5" t="inlineStr"/>
-      <c r="W7" t="inlineStr">
+      <c r="U7" s="5" t="inlineStr"/>
+      <c r="V7">
+        <f>IF(T7="Ne pas migrer","Ne pas migrer",IF(U7&lt;&gt;"",U7,IF(E7="Non","Ne pas migrer",S7)))</f>
+        <v/>
+      </c>
+      <c r="W7" s="5" t="inlineStr"/>
+      <c r="X7" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="X7" t="inlineStr">
+      <c r="Y7" t="inlineStr">
         <is>
           <t>À créer dans Zabbix</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>Spécificité à créer</t>
         </is>
       </c>
     </row>
@@ -7748,20 +9074,30 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G8,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G8,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G8,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T8" s="5" t="inlineStr"/>
-      <c r="U8">
-        <f>IF(T8&lt;&gt;"",T8,IF(E8="Non","Ne pas migrer",S8))</f>
+      <c r="T8">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A8,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A8,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A8,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V8" s="5" t="inlineStr"/>
-      <c r="W8" t="inlineStr">
+      <c r="U8" s="5" t="inlineStr"/>
+      <c r="V8">
+        <f>IF(T8="Ne pas migrer","Ne pas migrer",IF(U8&lt;&gt;"",U8,IF(E8="Non","Ne pas migrer",S8)))</f>
+        <v/>
+      </c>
+      <c r="W8" s="5" t="inlineStr"/>
+      <c r="X8" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="X8" t="inlineStr">
+      <c r="Y8" t="inlineStr">
         <is>
           <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>Spécificité à créer</t>
         </is>
       </c>
     </row>
@@ -7844,20 +9180,30 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G9,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G9,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G9,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T9" s="5" t="inlineStr"/>
-      <c r="U9">
-        <f>IF(T9&lt;&gt;"",T9,IF(E9="Non","Ne pas migrer",S9))</f>
+      <c r="T9">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A9,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A9,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A9,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V9" s="5" t="inlineStr"/>
-      <c r="W9" t="inlineStr">
+      <c r="U9" s="5" t="inlineStr"/>
+      <c r="V9">
+        <f>IF(T9="Ne pas migrer","Ne pas migrer",IF(U9&lt;&gt;"",U9,IF(E9="Non","Ne pas migrer",S9)))</f>
+        <v/>
+      </c>
+      <c r="W9" s="5" t="inlineStr"/>
+      <c r="X9" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="X9" t="inlineStr">
+      <c r="Y9" t="inlineStr">
         <is>
           <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>Spécificité à créer</t>
         </is>
       </c>
     </row>
@@ -7948,20 +9294,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G10,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G10,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G10,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T10" s="5" t="inlineStr"/>
-      <c r="U10">
-        <f>IF(T10&lt;&gt;"",T10,IF(E10="Non","Ne pas migrer",S10))</f>
+      <c r="T10">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A10,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A10,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A10,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V10" s="5" t="inlineStr"/>
-      <c r="W10" t="inlineStr">
+      <c r="U10" s="5" t="inlineStr"/>
+      <c r="V10">
+        <f>IF(T10="Ne pas migrer","Ne pas migrer",IF(U10&lt;&gt;"",U10,IF(E10="Non","Ne pas migrer",S10)))</f>
+        <v/>
+      </c>
+      <c r="W10" s="5" t="inlineStr"/>
+      <c r="X10" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="X10" t="inlineStr">
+      <c r="Y10" t="inlineStr">
         <is>
           <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>CPU utilization [system.cpu.util[snmp.cpu.util]]</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -8040,20 +9400,30 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G11,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G11,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G11,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T11" s="5" t="inlineStr"/>
-      <c r="U11">
-        <f>IF(T11&lt;&gt;"",T11,IF(E11="Non","Ne pas migrer",S11))</f>
+      <c r="T11">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A11,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A11,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A11,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V11" s="5" t="inlineStr"/>
-      <c r="W11" t="inlineStr">
+      <c r="U11" s="5" t="inlineStr"/>
+      <c r="V11">
+        <f>IF(T11="Ne pas migrer","Ne pas migrer",IF(U11&lt;&gt;"",U11,IF(E11="Non","Ne pas migrer",S11)))</f>
+        <v/>
+      </c>
+      <c r="W11" s="5" t="inlineStr"/>
+      <c r="X11" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="X11" t="inlineStr">
+      <c r="Y11" t="inlineStr">
         <is>
           <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>Spécificité à créer</t>
         </is>
       </c>
     </row>
@@ -8144,20 +9514,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G12,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G12,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G12,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T12" s="5" t="inlineStr"/>
-      <c r="U12">
-        <f>IF(T12&lt;&gt;"",T12,IF(E12="Non","Ne pas migrer",S12))</f>
+      <c r="T12">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A12,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A12,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A12,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V12" s="5" t="inlineStr"/>
-      <c r="W12" t="inlineStr">
+      <c r="U12" s="5" t="inlineStr"/>
+      <c r="V12">
+        <f>IF(T12="Ne pas migrer","Ne pas migrer",IF(U12&lt;&gt;"",U12,IF(E12="Non","Ne pas migrer",S12)))</f>
+        <v/>
+      </c>
+      <c r="W12" s="5" t="inlineStr"/>
+      <c r="X12" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="X12" t="inlineStr">
+      <c r="Y12" t="inlineStr">
         <is>
           <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>Memory utilization [vm.memory.util[snmp.vm.memory.util]]</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -8244,20 +9628,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G13,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G13,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G13,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T13" s="5" t="inlineStr"/>
-      <c r="U13">
-        <f>IF(T13&lt;&gt;"",T13,IF(E13="Non","Ne pas migrer",S13))</f>
+      <c r="T13">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A13,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A13,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A13,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V13" s="5" t="inlineStr"/>
-      <c r="W13" t="inlineStr">
+      <c r="U13" s="5" t="inlineStr"/>
+      <c r="V13">
+        <f>IF(T13="Ne pas migrer","Ne pas migrer",IF(U13&lt;&gt;"",U13,IF(E13="Non","Ne pas migrer",S13)))</f>
+        <v/>
+      </c>
+      <c r="W13" s="5" t="inlineStr"/>
+      <c r="X13" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="X13" t="inlineStr">
+      <c r="Y13" t="inlineStr">
         <is>
           <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>ICMP ping [icmpping] … (+2)</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -8348,20 +9746,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G14,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G14,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G14,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T14" s="5" t="inlineStr"/>
-      <c r="U14">
-        <f>IF(T14&lt;&gt;"",T14,IF(E14="Non","Ne pas migrer",S14))</f>
+      <c r="T14">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A14,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A14,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A14,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V14" s="5" t="inlineStr"/>
-      <c r="W14" t="inlineStr">
+      <c r="U14" s="5" t="inlineStr"/>
+      <c r="V14">
+        <f>IF(T14="Ne pas migrer","Ne pas migrer",IF(U14&lt;&gt;"",U14,IF(E14="Non","Ne pas migrer",S14)))</f>
+        <v/>
+      </c>
+      <c r="W14" s="5" t="inlineStr"/>
+      <c r="X14" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="X14" t="inlineStr">
+      <c r="Y14" t="inlineStr">
         <is>
           <t>Couvert dans Zabbix</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>Requests per second [apache.requests.rate] … (+1)</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -8452,20 +9864,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G15,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G15,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G15,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T15" s="5" t="inlineStr"/>
-      <c r="U15">
-        <f>IF(T15&lt;&gt;"",T15,IF(E15="Non","Ne pas migrer",S15))</f>
+      <c r="T15">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A15,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A15,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A15,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V15" s="5" t="inlineStr"/>
-      <c r="W15" t="inlineStr">
+      <c r="U15" s="5" t="inlineStr"/>
+      <c r="V15">
+        <f>IF(T15="Ne pas migrer","Ne pas migrer",IF(U15&lt;&gt;"",U15,IF(E15="Non","Ne pas migrer",S15)))</f>
+        <v/>
+      </c>
+      <c r="W15" s="5" t="inlineStr"/>
+      <c r="X15" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="X15" t="inlineStr">
+      <c r="Y15" t="inlineStr">
         <is>
           <t>Couvert dans Zabbix</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>CPU utilization [system.cpu.util[snmp.cpu.util]]</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -8556,20 +9982,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G16,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G16,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G16,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T16" s="5" t="inlineStr"/>
-      <c r="U16">
-        <f>IF(T16&lt;&gt;"",T16,IF(E16="Non","Ne pas migrer",S16))</f>
+      <c r="T16">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A16,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A16,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A16,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V16" s="5" t="inlineStr"/>
-      <c r="W16" t="inlineStr">
+      <c r="U16" s="5" t="inlineStr"/>
+      <c r="V16">
+        <f>IF(T16="Ne pas migrer","Ne pas migrer",IF(U16&lt;&gt;"",U16,IF(E16="Non","Ne pas migrer",S16)))</f>
+        <v/>
+      </c>
+      <c r="W16" s="5" t="inlineStr"/>
+      <c r="X16" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="X16" t="inlineStr">
+      <c r="Y16" t="inlineStr">
         <is>
           <t>Couvert dans Zabbix</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>{#FSNAME}: Space utilization [vfs.fs.pused[storageUsedPercentage.{#SNMPINDEX}]] (LLD)</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -8664,20 +10104,30 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G17,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G17,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G17,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T17" s="5" t="inlineStr"/>
-      <c r="U17">
-        <f>IF(T17&lt;&gt;"",T17,IF(E17="Non","Ne pas migrer",S17))</f>
+      <c r="T17">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A17,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A17,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A17,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V17" s="5" t="inlineStr"/>
-      <c r="W17" t="inlineStr">
+      <c r="U17" s="5" t="inlineStr"/>
+      <c r="V17">
+        <f>IF(T17="Ne pas migrer","Ne pas migrer",IF(U17&lt;&gt;"",U17,IF(E17="Non","Ne pas migrer",S17)))</f>
+        <v/>
+      </c>
+      <c r="W17" s="5" t="inlineStr"/>
+      <c r="X17" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="X17" t="inlineStr">
+      <c r="Y17" t="inlineStr">
         <is>
           <t>Template à lier</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr"/>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>Template standard à importer dans Zabbix</t>
         </is>
       </c>
     </row>
@@ -8768,20 +10218,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G18,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G18,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G18,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T18" s="5" t="inlineStr"/>
-      <c r="U18">
-        <f>IF(T18&lt;&gt;"",T18,IF(E18="Non","Ne pas migrer",S18))</f>
+      <c r="T18">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A18,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A18,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A18,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V18" s="5" t="inlineStr"/>
-      <c r="W18" t="inlineStr">
+      <c r="U18" s="5" t="inlineStr"/>
+      <c r="V18">
+        <f>IF(T18="Ne pas migrer","Ne pas migrer",IF(U18&lt;&gt;"",U18,IF(E18="Non","Ne pas migrer",S18)))</f>
+        <v/>
+      </c>
+      <c r="W18" s="5" t="inlineStr"/>
+      <c r="X18" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="X18" t="inlineStr">
+      <c r="Y18" t="inlineStr">
         <is>
           <t>Couvert dans Zabbix</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>Memory utilization [vm.memory.util[snmp.vm.memory.util]]</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -8872,20 +10336,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G19,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G19,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G19,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T19" s="5" t="inlineStr"/>
-      <c r="U19">
-        <f>IF(T19&lt;&gt;"",T19,IF(E19="Non","Ne pas migrer",S19))</f>
+      <c r="T19">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A19,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A19,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A19,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V19" s="5" t="inlineStr"/>
-      <c r="W19" t="inlineStr">
+      <c r="U19" s="5" t="inlineStr"/>
+      <c r="V19">
+        <f>IF(T19="Ne pas migrer","Ne pas migrer",IF(U19&lt;&gt;"",U19,IF(E19="Non","Ne pas migrer",S19)))</f>
+        <v/>
+      </c>
+      <c r="W19" s="5" t="inlineStr"/>
+      <c r="X19" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="X19" t="inlineStr">
+      <c r="Y19" t="inlineStr">
         <is>
           <t>Non migré (décision)</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>Memory utilization [vm.memory.util[snmp.vm.memory.util]]</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>Non migré</t>
         </is>
       </c>
     </row>
@@ -8972,20 +10450,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G20,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G20,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G20,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T20" s="5" t="inlineStr"/>
-      <c r="U20">
-        <f>IF(T20&lt;&gt;"",T20,IF(E20="Non","Ne pas migrer",S20))</f>
+      <c r="T20">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A20,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A20,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A20,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V20" s="5" t="inlineStr"/>
-      <c r="W20" t="inlineStr">
+      <c r="U20" s="5" t="inlineStr"/>
+      <c r="V20">
+        <f>IF(T20="Ne pas migrer","Ne pas migrer",IF(U20&lt;&gt;"",U20,IF(E20="Non","Ne pas migrer",S20)))</f>
+        <v/>
+      </c>
+      <c r="W20" s="5" t="inlineStr"/>
+      <c r="X20" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="X20" t="inlineStr">
+      <c r="Y20" t="inlineStr">
         <is>
           <t>Couvert dans Zabbix</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>ICMP ping [icmpping] … (+2)</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -9076,20 +10568,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G21,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G21,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G21,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T21" s="5" t="inlineStr"/>
-      <c r="U21">
-        <f>IF(T21&lt;&gt;"",T21,IF(E21="Non","Ne pas migrer",S21))</f>
+      <c r="T21">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A21,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A21,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A21,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V21" s="5" t="inlineStr"/>
-      <c r="W21" t="inlineStr">
+      <c r="U21" s="5" t="inlineStr"/>
+      <c r="V21">
+        <f>IF(T21="Ne pas migrer","Ne pas migrer",IF(U21&lt;&gt;"",U21,IF(E21="Non","Ne pas migrer",S21)))</f>
+        <v/>
+      </c>
+      <c r="W21" s="5" t="inlineStr"/>
+      <c r="X21" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="X21" t="inlineStr">
+      <c r="Y21" t="inlineStr">
         <is>
           <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>Requests per second [apache.requests.rate] … (+1)</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -9180,20 +10686,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G22,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G22,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G22,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T22" s="5" t="inlineStr"/>
-      <c r="U22">
-        <f>IF(T22&lt;&gt;"",T22,IF(E22="Non","Ne pas migrer",S22))</f>
+      <c r="T22">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A22,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A22,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A22,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V22" s="5" t="inlineStr"/>
-      <c r="W22" t="inlineStr">
+      <c r="U22" s="5" t="inlineStr"/>
+      <c r="V22">
+        <f>IF(T22="Ne pas migrer","Ne pas migrer",IF(U22&lt;&gt;"",U22,IF(E22="Non","Ne pas migrer",S22)))</f>
+        <v/>
+      </c>
+      <c r="W22" s="5" t="inlineStr"/>
+      <c r="X22" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="X22" t="inlineStr">
+      <c r="Y22" t="inlineStr">
         <is>
           <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>CPU utilization [system.cpu.util[snmp.cpu.util]]</t>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -9284,20 +10804,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G23,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G23,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G23,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T23" s="5" t="inlineStr"/>
-      <c r="U23">
-        <f>IF(T23&lt;&gt;"",T23,IF(E23="Non","Ne pas migrer",S23))</f>
+      <c r="T23">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A23,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A23,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A23,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V23" s="5" t="inlineStr"/>
-      <c r="W23" t="inlineStr">
+      <c r="U23" s="5" t="inlineStr"/>
+      <c r="V23">
+        <f>IF(T23="Ne pas migrer","Ne pas migrer",IF(U23&lt;&gt;"",U23,IF(E23="Non","Ne pas migrer",S23)))</f>
+        <v/>
+      </c>
+      <c r="W23" s="5" t="inlineStr"/>
+      <c r="X23" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="X23" t="inlineStr">
+      <c r="Y23" t="inlineStr">
         <is>
           <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>{#FSNAME}: Space utilization [vfs.fs.pused[storageUsedPercentage.{#SNMPINDEX}]] (LLD)</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -9392,20 +10926,30 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G24,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G24,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G24,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T24" s="5" t="inlineStr"/>
-      <c r="U24">
-        <f>IF(T24&lt;&gt;"",T24,IF(E24="Non","Ne pas migrer",S24))</f>
+      <c r="T24">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A24,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A24,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A24,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V24" s="5" t="inlineStr"/>
-      <c r="W24" t="inlineStr">
+      <c r="U24" s="5" t="inlineStr"/>
+      <c r="V24">
+        <f>IF(T24="Ne pas migrer","Ne pas migrer",IF(U24&lt;&gt;"",U24,IF(E24="Non","Ne pas migrer",S24)))</f>
+        <v/>
+      </c>
+      <c r="W24" s="5" t="inlineStr"/>
+      <c r="X24" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="X24" t="inlineStr">
+      <c r="Y24" t="inlineStr">
         <is>
           <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
+      <c r="Z24" t="inlineStr"/>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>Template standard à importer dans Zabbix</t>
         </is>
       </c>
     </row>
@@ -9496,20 +11040,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G25,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G25,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G25,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T25" s="5" t="inlineStr"/>
-      <c r="U25">
-        <f>IF(T25&lt;&gt;"",T25,IF(E25="Non","Ne pas migrer",S25))</f>
+      <c r="T25">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A25,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A25,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A25,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V25" s="5" t="inlineStr"/>
-      <c r="W25" t="inlineStr">
+      <c r="U25" s="5" t="inlineStr"/>
+      <c r="V25">
+        <f>IF(T25="Ne pas migrer","Ne pas migrer",IF(U25&lt;&gt;"",U25,IF(E25="Non","Ne pas migrer",S25)))</f>
+        <v/>
+      </c>
+      <c r="W25" s="5" t="inlineStr"/>
+      <c r="X25" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="X25" t="inlineStr">
+      <c r="Y25" t="inlineStr">
         <is>
           <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>Memory utilization [vm.memory.util[snmp.vm.memory.util]]</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -9596,20 +11154,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G26,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G26,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G26,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T26" s="5" t="inlineStr"/>
-      <c r="U26">
-        <f>IF(T26&lt;&gt;"",T26,IF(E26="Non","Ne pas migrer",S26))</f>
+      <c r="T26">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A26,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A26,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A26,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V26" s="5" t="inlineStr"/>
-      <c r="W26" t="inlineStr">
+      <c r="U26" s="5" t="inlineStr"/>
+      <c r="V26">
+        <f>IF(T26="Ne pas migrer","Ne pas migrer",IF(U26&lt;&gt;"",U26,IF(E26="Non","Ne pas migrer",S26)))</f>
+        <v/>
+      </c>
+      <c r="W26" s="5" t="inlineStr"/>
+      <c r="X26" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="X26" t="inlineStr">
+      <c r="Y26" t="inlineStr">
         <is>
           <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>ICMP ping [icmpping] … (+2)</t>
+        </is>
+      </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -9700,20 +11272,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G27,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G27,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G27,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T27" s="5" t="inlineStr"/>
-      <c r="U27">
-        <f>IF(T27&lt;&gt;"",T27,IF(E27="Non","Ne pas migrer",S27))</f>
+      <c r="T27">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A27,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A27,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A27,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V27" s="5" t="inlineStr"/>
-      <c r="W27" t="inlineStr">
+      <c r="U27" s="5" t="inlineStr"/>
+      <c r="V27">
+        <f>IF(T27="Ne pas migrer","Ne pas migrer",IF(U27&lt;&gt;"",U27,IF(E27="Non","Ne pas migrer",S27)))</f>
+        <v/>
+      </c>
+      <c r="W27" s="5" t="inlineStr"/>
+      <c r="X27" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="X27" t="inlineStr">
+      <c r="Y27" t="inlineStr">
         <is>
           <t>Template à lier</t>
+        </is>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>CPU utilization [system.cpu.util[snmp.cpu.util]]</t>
+        </is>
+      </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -9804,20 +11390,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G28,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G28,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G28,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T28" s="5" t="inlineStr"/>
-      <c r="U28">
-        <f>IF(T28&lt;&gt;"",T28,IF(E28="Non","Ne pas migrer",S28))</f>
+      <c r="T28">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A28,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A28,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A28,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V28" s="5" t="inlineStr"/>
-      <c r="W28" t="inlineStr">
+      <c r="U28" s="5" t="inlineStr"/>
+      <c r="V28">
+        <f>IF(T28="Ne pas migrer","Ne pas migrer",IF(U28&lt;&gt;"",U28,IF(E28="Non","Ne pas migrer",S28)))</f>
+        <v/>
+      </c>
+      <c r="W28" s="5" t="inlineStr"/>
+      <c r="X28" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="X28" t="inlineStr">
+      <c r="Y28" t="inlineStr">
         <is>
           <t>Template à lier</t>
+        </is>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>{#FSNAME}: Space utilization [vfs.fs.pused[storageUsedPercentage.{#SNMPINDEX}]] (LLD)</t>
+        </is>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -9900,20 +11500,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G29,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G29,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G29,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T29" s="5" t="inlineStr"/>
-      <c r="U29">
-        <f>IF(T29&lt;&gt;"",T29,IF(E29="Non","Ne pas migrer",S29))</f>
+      <c r="T29">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A29,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A29,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A29,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V29" s="5" t="inlineStr"/>
-      <c r="W29" t="inlineStr">
+      <c r="U29" s="5" t="inlineStr"/>
+      <c r="V29">
+        <f>IF(T29="Ne pas migrer","Ne pas migrer",IF(U29&lt;&gt;"",U29,IF(E29="Non","Ne pas migrer",S29)))</f>
+        <v/>
+      </c>
+      <c r="W29" s="5" t="inlineStr"/>
+      <c r="X29" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="X29" t="inlineStr">
+      <c r="Y29" t="inlineStr">
         <is>
           <t>Couvert dans Zabbix</t>
+        </is>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>State of service "{#SERVICE.NAME}" [service.info["{#SERVICE.NAME}",state]] (LLD)</t>
+        </is>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -10004,20 +11618,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G30,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G30,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G30,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T30" s="5" t="inlineStr"/>
-      <c r="U30">
-        <f>IF(T30&lt;&gt;"",T30,IF(E30="Non","Ne pas migrer",S30))</f>
+      <c r="T30">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A30,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A30,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A30,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V30" s="5" t="inlineStr"/>
-      <c r="W30" t="inlineStr">
+      <c r="U30" s="5" t="inlineStr"/>
+      <c r="V30">
+        <f>IF(T30="Ne pas migrer","Ne pas migrer",IF(U30&lt;&gt;"",U30,IF(E30="Non","Ne pas migrer",S30)))</f>
+        <v/>
+      </c>
+      <c r="W30" s="5" t="inlineStr"/>
+      <c r="X30" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="X30" t="inlineStr">
+      <c r="Y30" t="inlineStr">
         <is>
           <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>CPU utilization [system.cpu.util[snmp.cpu.util]]</t>
+        </is>
+      </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -10108,20 +11736,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G31,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G31,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G31,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T31" s="5" t="inlineStr"/>
-      <c r="U31">
-        <f>IF(T31&lt;&gt;"",T31,IF(E31="Non","Ne pas migrer",S31))</f>
+      <c r="T31">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A31,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A31,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A31,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V31" s="5" t="inlineStr"/>
-      <c r="W31" t="inlineStr">
+      <c r="U31" s="5" t="inlineStr"/>
+      <c r="V31">
+        <f>IF(T31="Ne pas migrer","Ne pas migrer",IF(U31&lt;&gt;"",U31,IF(E31="Non","Ne pas migrer",S31)))</f>
+        <v/>
+      </c>
+      <c r="W31" s="5" t="inlineStr"/>
+      <c r="X31" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="X31" t="inlineStr">
+      <c r="Y31" t="inlineStr">
         <is>
           <t>Hôte absent de Zabbix</t>
+        </is>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>{#FSNAME}: Space utilization [vfs.fs.pused[storageUsedPercentage.{#SNMPINDEX}]] (LLD)</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -10200,20 +11842,30 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G32,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G32,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G32,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T32" s="5" t="inlineStr"/>
-      <c r="U32">
-        <f>IF(T32&lt;&gt;"",T32,IF(E32="Non","Ne pas migrer",S32))</f>
+      <c r="T32">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A32,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A32,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A32,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V32" s="5" t="inlineStr"/>
-      <c r="W32" t="inlineStr">
+      <c r="U32" s="5" t="inlineStr"/>
+      <c r="V32">
+        <f>IF(T32="Ne pas migrer","Ne pas migrer",IF(U32&lt;&gt;"",U32,IF(E32="Non","Ne pas migrer",S32)))</f>
+        <v/>
+      </c>
+      <c r="W32" s="5" t="inlineStr"/>
+      <c r="X32" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="X32" t="inlineStr">
+      <c r="Y32" t="inlineStr">
         <is>
           <t>Non migré (décision)</t>
+        </is>
+      </c>
+      <c r="Z32" t="inlineStr"/>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>Non migré</t>
         </is>
       </c>
     </row>
@@ -10304,20 +11956,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G33,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G33,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G33,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T33" s="5" t="inlineStr"/>
-      <c r="U33">
-        <f>IF(T33&lt;&gt;"",T33,IF(E33="Non","Ne pas migrer",S33))</f>
+      <c r="T33">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A33,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A33,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A33,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V33" s="5" t="inlineStr"/>
-      <c r="W33" t="inlineStr">
+      <c r="U33" s="5" t="inlineStr"/>
+      <c r="V33">
+        <f>IF(T33="Ne pas migrer","Ne pas migrer",IF(U33&lt;&gt;"",U33,IF(E33="Non","Ne pas migrer",S33)))</f>
+        <v/>
+      </c>
+      <c r="W33" s="5" t="inlineStr"/>
+      <c r="X33" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="X33" t="inlineStr">
+      <c r="Y33" t="inlineStr">
         <is>
           <t>Non migré (décision)</t>
+        </is>
+      </c>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>{#SENSOR_INFO}: Temperature [sensor.temp.value[ciscoEnvMonTemperatureValue.{#SNMPINDEX}]] (LLD)</t>
+        </is>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>Non migré</t>
         </is>
       </c>
     </row>
@@ -10408,20 +12074,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G34,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G34,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G34,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T34" s="5" t="inlineStr"/>
-      <c r="U34">
-        <f>IF(T34&lt;&gt;"",T34,IF(E34="Non","Ne pas migrer",S34))</f>
+      <c r="T34">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A34,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A34,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A34,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V34" s="5" t="inlineStr"/>
-      <c r="W34" t="inlineStr">
+      <c r="U34" s="5" t="inlineStr"/>
+      <c r="V34">
+        <f>IF(T34="Ne pas migrer","Ne pas migrer",IF(U34&lt;&gt;"",U34,IF(E34="Non","Ne pas migrer",S34)))</f>
+        <v/>
+      </c>
+      <c r="W34" s="5" t="inlineStr"/>
+      <c r="X34" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="X34" t="inlineStr">
+      <c r="Y34" t="inlineStr">
         <is>
           <t>À créer dans Zabbix</t>
+        </is>
+      </c>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>{#SENSOR_INFO}: Temperature [sensor.temp.value[ciscoEnvMonTemperatureValue.{#SNMPINDEX}]] (LLD)</t>
+        </is>
+      </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -10512,20 +12192,34 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G35,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G35,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G35,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T35" s="5" t="inlineStr"/>
-      <c r="U35">
-        <f>IF(T35&lt;&gt;"",T35,IF(E35="Non","Ne pas migrer",S35))</f>
+      <c r="T35">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A35,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A35,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A35,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V35" s="5" t="inlineStr"/>
-      <c r="W35" t="inlineStr">
+      <c r="U35" s="5" t="inlineStr"/>
+      <c r="V35">
+        <f>IF(T35="Ne pas migrer","Ne pas migrer",IF(U35&lt;&gt;"",U35,IF(E35="Non","Ne pas migrer",S35)))</f>
+        <v/>
+      </c>
+      <c r="W35" s="5" t="inlineStr"/>
+      <c r="X35" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="X35" t="inlineStr">
+      <c r="Y35" t="inlineStr">
         <is>
           <t>À créer dans Zabbix</t>
+        </is>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>Interface {#IFNAME}: Bits received [net.if.in[ifHCInOctets.{#SNMPINDEX}]] (LLD)</t>
+        </is>
+      </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
         </is>
       </c>
     </row>
@@ -10608,25 +12302,39 @@
         <f>IFERROR(IF(INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G36,'Matrice templates services'!$A$2:$A$23,0))&lt;&gt;"",INDEX('Matrice templates services'!$Y$2:$Y$23,MATCH($G36,'Matrice templates services'!$A$2:$A$23,0)),INDEX('Matrice templates services'!$X$2:$X$23,MATCH($G36,'Matrice templates services'!$A$2:$A$23,0))),"")</f>
         <v/>
       </c>
-      <c r="T36" s="5" t="inlineStr"/>
-      <c r="U36">
-        <f>IF(T36&lt;&gt;"",T36,IF(E36="Non","Ne pas migrer",S36))</f>
+      <c r="T36">
+        <f>IFERROR(IF(INDEX('Hôtes'!$P$2:$P$10,MATCH($A36,'Hôtes'!$A$2:$A$10,0))&lt;&gt;"",INDEX('Hôtes'!$P$2:$P$10,MATCH($A36,'Hôtes'!$A$2:$A$10,0)),INDEX('Hôtes'!$O$2:$O$10,MATCH($A36,'Hôtes'!$A$2:$A$10,0))),"")</f>
         <v/>
       </c>
-      <c r="V36" s="5" t="inlineStr"/>
-      <c r="W36" t="inlineStr">
+      <c r="U36" s="5" t="inlineStr"/>
+      <c r="V36">
+        <f>IF(T36="Ne pas migrer","Ne pas migrer",IF(U36&lt;&gt;"",U36,IF(E36="Non","Ne pas migrer",S36)))</f>
+        <v/>
+      </c>
+      <c r="W36" s="5" t="inlineStr"/>
+      <c r="X36" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="X36" t="inlineStr">
+      <c r="Y36" t="inlineStr">
         <is>
           <t>Hôte absent de Zabbix</t>
         </is>
       </c>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>ICMP ping [icmpping] … (+2)</t>
+        </is>
+      </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>Couvert par un item standard</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X36"/>
+  <autoFilter ref="A1:AA36"/>
   <conditionalFormatting sqref="R2:R36">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>R2="Migrer (template natif)"</formula>
@@ -10719,40 +12427,125 @@
       <formula>U2="Migrer"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X2:X36">
+  <conditionalFormatting sqref="V2:V36">
     <cfRule type="expression" priority="29" dxfId="0">
-      <formula>X2="Présent – templates OK"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="30" dxfId="0">
-      <formula>X2="Couvert dans Zabbix"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="31" dxfId="4">
-      <formula>X2="Présent – templates à lier"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="32" dxfId="4">
-      <formula>X2="Template à lier"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="33" dxfId="1">
-      <formula>X2="Présent"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="34" dxfId="6">
-      <formula>X2="Absent de Zabbix"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="35" dxfId="6">
-      <formula>X2="Hôte absent de Zabbix"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="36" dxfId="2">
-      <formula>X2="À créer dans Zabbix"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="37" dxfId="3">
-      <formula>X2="Non migré (décision)"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="38" dxfId="6">
-      <formula>X2="Non (à importer)"</formula>
+      <formula>V2="Migrer (template natif)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="30" dxfId="1">
+      <formula>V2="Migrer (adapter)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="31" dxfId="2">
+      <formula>V2="Migrer (développer)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="32" dxfId="3">
+      <formula>V2="Ne pas migrer"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="33" dxfId="4">
+      <formula>V2="À analyser"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="34" dxfId="5">
+      <formula>V2="Hérité (pas d'action directe)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="35" dxfId="0">
+      <formula>V2="Migrer"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Y2:Y36">
+    <cfRule type="expression" priority="36" dxfId="0">
+      <formula>Y2="Présent – templates OK"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="37" dxfId="0">
+      <formula>Y2="Couvert dans Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="38" dxfId="4">
+      <formula>Y2="Présent – templates à lier"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="39" dxfId="4">
+      <formula>Y2="Template à lier"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="40" dxfId="1">
+      <formula>Y2="Présent"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="41" dxfId="6">
+      <formula>Y2="Absent de Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="42" dxfId="6">
+      <formula>Y2="Hôte absent de Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="43" dxfId="2">
+      <formula>Y2="À créer dans Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="44" dxfId="3">
+      <formula>Y2="Non migré (décision)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="45" dxfId="6">
+      <formula>Y2="Non (à importer)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="46" dxfId="0">
+      <formula>Y2="Couvert par un item standard"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="47" dxfId="4">
+      <formula>Y2="Template standard sans item correspondant"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="48" dxfId="1">
+      <formula>Y2="Template standard à importer dans Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="49" dxfId="2">
+      <formula>Y2="Spécificité à créer"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="50" dxfId="3">
+      <formula>Y2="Non migré"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AA2:AA36">
+    <cfRule type="expression" priority="51" dxfId="0">
+      <formula>AA2="Présent – templates OK"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="52" dxfId="0">
+      <formula>AA2="Couvert dans Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="53" dxfId="4">
+      <formula>AA2="Présent – templates à lier"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="54" dxfId="4">
+      <formula>AA2="Template à lier"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="55" dxfId="1">
+      <formula>AA2="Présent"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="56" dxfId="6">
+      <formula>AA2="Absent de Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="57" dxfId="6">
+      <formula>AA2="Hôte absent de Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="58" dxfId="2">
+      <formula>AA2="À créer dans Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="59" dxfId="3">
+      <formula>AA2="Non migré (décision)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="60" dxfId="6">
+      <formula>AA2="Non (à importer)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="61" dxfId="0">
+      <formula>AA2="Couvert par un item standard"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="62" dxfId="4">
+      <formula>AA2="Template standard sans item correspondant"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="63" dxfId="1">
+      <formula>AA2="Template standard à importer dans Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="64" dxfId="2">
+      <formula>AA2="Spécificité à créer"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="65" dxfId="3">
+      <formula>AA2="Non migré"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="T2:T36" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Décision" error="Choisir une valeur dans la liste" type="list">
+    <dataValidation sqref="U2:U36" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Décision" error="Choisir une valeur dans la liste" type="list">
       <formula1>"Migrer (template natif),Migrer (adapter),Migrer (développer),Ne pas migrer,À analyser,Hérité (pas d'action directe)"</formula1>
     </dataValidation>
   </dataValidations>
@@ -12347,6 +14140,21 @@
     <cfRule type="expression" priority="10" dxfId="6">
       <formula>E2="Non (à importer)"</formula>
     </cfRule>
+    <cfRule type="expression" priority="11" dxfId="0">
+      <formula>E2="Couvert par un item standard"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="12" dxfId="4">
+      <formula>E2="Template standard sans item correspondant"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="13" dxfId="1">
+      <formula>E2="Template standard à importer dans Zabbix"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" dxfId="2">
+      <formula>E2="Spécificité à créer"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="15" dxfId="3">
+      <formula>E2="Non migré"</formula>
+    </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>